<commit_message>
Regenerate user-story mapping with R1-R6 (70 -> 76 items)
Keeps the spreadsheet in sync with ROADMAP.md's new Risk, compliance &
real-world operations section rather than letting it drift. The
readable Word doc was regenerated from the same source in the same
pass (untracked, per convention).
</commit_message>
<xml_diff>
--- a/docs/LMX_OS_Roadmap_User_Stories.xlsx
+++ b/docs/LMX_OS_Roadmap_User_Stories.xlsx
@@ -11,7 +11,7 @@
     <sheet xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" name="User Stories" sheetId="2" state="visible" r:id="rId2"/>
   </sheets>
   <definedNames>
-    <definedName name="_xlnm._FilterDatabase" localSheetId="1" hidden="1">'User Stories'!$A$1:$F$71</definedName>
+    <definedName name="_xlnm._FilterDatabase" localSheetId="1" hidden="1">'User Stories'!$A$1:$F$77</definedName>
   </definedNames>
   <calcPr calcId="124519" fullCalcOnLoad="1"/>
 </workbook>
@@ -620,7 +620,7 @@
     <outlinePr summaryBelow="1" summaryRight="1"/>
     <pageSetUpPr/>
   </sheetPr>
-  <dimension ref="A1:F71"/>
+  <dimension ref="A1:F77"/>
   <sheetFormatPr baseColWidth="8" defaultRowHeight="15"/>
   <cols>
     <col width="7" customWidth="1" min="1" max="1"/>
@@ -826,113 +826,113 @@
     <row r="7">
       <c r="A7" s="7" t="inlineStr">
         <is>
-          <t>E1</t>
+          <t>R1</t>
         </is>
       </c>
       <c r="B7" s="8" t="inlineStr">
         <is>
-          <t>Core backend</t>
+          <t>Risk &amp; compliance</t>
         </is>
       </c>
       <c r="C7" s="8" t="inlineStr">
         <is>
-          <t>Verify Google Route Optimization against a live project</t>
+          <t>Insurance &amp; liability plan</t>
         </is>
       </c>
       <c r="D7" s="7" t="inlineStr">
         <is>
-          <t>Open</t>
+          <t>Open - gates Phase 9</t>
         </is>
       </c>
       <c r="E7" s="8" t="inlineStr">
         <is>
-          <t>Phase 4</t>
+          <t>Start now (business/legal)</t>
         </is>
       </c>
       <c r="F7" s="8" t="inlineStr">
         <is>
-          <t>As a hub dispatcher relying on the optimizer, I want the Google Route Optimization integration verified against a real API call, so that I can trust the routes it proposes instead of an unverified request/response mapping.</t>
+          <t>As LMX leadership, I want commercial auto, cargo, and general liability coverage in place before drivers carry real packages, so that a single accident or lost shipment is an insured event rather than a company-ending liability.</t>
         </is>
       </c>
     </row>
     <row r="8">
       <c r="A8" s="5" t="inlineStr">
         <is>
-          <t>E2</t>
+          <t>R2</t>
         </is>
       </c>
       <c r="B8" s="6" t="inlineStr">
         <is>
-          <t>Core backend</t>
+          <t>Risk &amp; compliance</t>
         </is>
       </c>
       <c r="C8" s="6" t="inlineStr">
         <is>
-          <t>Tune SLA_TIER_SKIP_PENALTY values</t>
+          <t>Driver background checks &amp; MVR screening</t>
         </is>
       </c>
       <c r="D8" s="5" t="inlineStr">
         <is>
-          <t>Open</t>
+          <t>Open - gates Phase 9</t>
         </is>
       </c>
       <c r="E8" s="6" t="inlineStr">
         <is>
-          <t>Phase 4 / I5</t>
+          <t>Start now (business/legal)</t>
         </is>
       </c>
       <c r="F8" s="6" t="inlineStr">
         <is>
-          <t>As a hub dispatcher, I want the SLA tier skip penalties tuned to real route economics, so that the optimizer's tier prioritization reflects actual cost tradeoffs instead of a placeholder ordering.</t>
+          <t>As LMX leadership, I want every driver background-checked and their motor-vehicle record screened before their first shift, so that we know a driver is safe to put on the road - document expiry tracking alone doesn't tell us that.</t>
         </is>
       </c>
     </row>
     <row r="9">
       <c r="A9" s="7" t="inlineStr">
         <is>
-          <t>E3</t>
+          <t>R3</t>
         </is>
       </c>
       <c r="B9" s="8" t="inlineStr">
         <is>
-          <t>Core backend</t>
+          <t>Risk &amp; compliance</t>
         </is>
       </c>
       <c r="C9" s="8" t="inlineStr">
         <is>
-          <t>Confirm real Epicor payload field names</t>
+          <t>Privacy policy &amp; data-handling/retention policy</t>
         </is>
       </c>
       <c r="D9" s="7" t="inlineStr">
         <is>
-          <t>Open</t>
+          <t>Open - gates Phase 9</t>
         </is>
       </c>
       <c r="E9" s="8" t="inlineStr">
         <is>
-          <t>Phase 4 (needs B2)</t>
+          <t>Start now (business/legal)</t>
         </is>
       </c>
       <c r="F9" s="8" t="inlineStr">
         <is>
-          <t>As the engineer integrating with a client's Epicor system, I want the real payload field names confirmed against a live tenant, so that orders ingest correctly instead of failing on a guessed schema.</t>
+          <t>As a customer whose name, address, and phone number LMX stores, I want a published policy saying what happens to my data and how I can have it deleted, so that my information is handled accountably - and so LMX can answer an enterprise client's security questionnaire.</t>
         </is>
       </c>
     </row>
     <row r="10">
       <c r="A10" s="5" t="inlineStr">
         <is>
-          <t>E4</t>
+          <t>R4</t>
         </is>
       </c>
       <c r="B10" s="6" t="inlineStr">
         <is>
-          <t>Core backend</t>
+          <t>Risk &amp; compliance</t>
         </is>
       </c>
       <c r="C10" s="6" t="inlineStr">
         <is>
-          <t>Verify the batch-hold 4-question decision logic</t>
+          <t>Driver document upload pipeline</t>
         </is>
       </c>
       <c r="D10" s="5" t="inlineStr">
@@ -942,29 +942,29 @@
       </c>
       <c r="E10" s="6" t="inlineStr">
         <is>
-          <t>Phase 4 (needs B3)</t>
+          <t>Phase 6 (with A3)</t>
         </is>
       </c>
       <c r="F10" s="6" t="inlineStr">
         <is>
-          <t>As a hub dispatcher, I want the batch-hold decision logic verified against the canonical spec, so that commingling decisions match the intended design rather than a reconstructed interpretation.</t>
+          <t>As LMX's onboarding staff, I want drivers to upload real license and insurance documents through the app, so that compliance evidence is a verified file on record rather than whatever text string was typed into the field.</t>
         </is>
       </c>
     </row>
     <row r="11">
       <c r="A11" s="7" t="inlineStr">
         <is>
-          <t>E5</t>
+          <t>R5</t>
         </is>
       </c>
       <c r="B11" s="8" t="inlineStr">
         <is>
-          <t>Core backend</t>
+          <t>Risk &amp; compliance</t>
         </is>
       </c>
       <c r="C11" s="8" t="inlineStr">
         <is>
-          <t>Recalibrate SLA hold-window minutes</t>
+          <t>Failed-delivery / redelivery workflow</t>
         </is>
       </c>
       <c r="D11" s="7" t="inlineStr">
@@ -974,29 +974,29 @@
       </c>
       <c r="E11" s="8" t="inlineStr">
         <is>
-          <t>Phase 4 / I5</t>
+          <t>Phase 4</t>
         </is>
       </c>
       <c r="F11" s="8" t="inlineStr">
         <is>
-          <t>As a hub dispatcher, I want the SLA hold-window minutes recalibrated from real Hub 1 data, so that orders are held just long enough to batch efficiently without risking an SLA breach.</t>
+          <t>As a hub dispatcher facing a refused package, wrong address, or closed shop, I want a defined path for what happens next - redelivery, client notification, billing adjustment - so that a failed order gets resolved instead of sitting in a dead-end status forever.</t>
         </is>
       </c>
     </row>
     <row r="12">
       <c r="A12" s="5" t="inlineStr">
         <is>
-          <t>E6</t>
+          <t>R6</t>
         </is>
       </c>
       <c r="B12" s="6" t="inlineStr">
         <is>
-          <t>Core backend</t>
+          <t>Risk &amp; compliance</t>
         </is>
       </c>
       <c r="C12" s="6" t="inlineStr">
         <is>
-          <t>Confirm Learning Loop flag-type naming convention</t>
+          <t>Hub closure / holiday calendar</t>
         </is>
       </c>
       <c r="D12" s="5" t="inlineStr">
@@ -1011,14 +1011,14 @@
       </c>
       <c r="F12" s="6" t="inlineStr">
         <is>
-          <t>As the engineer building the annotation loop, I want the flag-type naming convention signed off by a driver-app stakeholder, so that the contract between driver annotations and the Learning Loop isn't just an internal guess.</t>
+          <t>As a hub ops manager, I want to mark days the hub isn't operating, so that the nightly learning job and the dispatch optimizer don't plan routes for a hub that's closed for a holiday or weather event.</t>
         </is>
       </c>
     </row>
     <row r="13">
       <c r="A13" s="7" t="inlineStr">
         <is>
-          <t>E7</t>
+          <t>E1</t>
         </is>
       </c>
       <c r="B13" s="8" t="inlineStr">
@@ -1028,12 +1028,12 @@
       </c>
       <c r="C13" s="8" t="inlineStr">
         <is>
-          <t>Wire a real scheduler for the Learning Loop's nightly job</t>
-        </is>
-      </c>
-      <c r="D13" s="9" t="inlineStr">
-        <is>
-          <t>Done</t>
+          <t>Verify Google Route Optimization against a live project</t>
+        </is>
+      </c>
+      <c r="D13" s="7" t="inlineStr">
+        <is>
+          <t>Open</t>
         </is>
       </c>
       <c r="E13" s="8" t="inlineStr">
@@ -1043,14 +1043,14 @@
       </c>
       <c r="F13" s="8" t="inlineStr">
         <is>
-          <t>As a hub, I want the Learning Loop's nightly detection job to run automatically on schedule, so that rule proposals get generated every night without anyone manually triggering it.</t>
+          <t>As a hub dispatcher relying on the optimizer, I want the Google Route Optimization integration verified against a real API call, so that I can trust the routes it proposes instead of an unverified request/response mapping.</t>
         </is>
       </c>
     </row>
     <row r="14">
       <c r="A14" s="5" t="inlineStr">
         <is>
-          <t>E8</t>
+          <t>E2</t>
         </is>
       </c>
       <c r="B14" s="6" t="inlineStr">
@@ -1060,29 +1060,29 @@
       </c>
       <c r="C14" s="6" t="inlineStr">
         <is>
-          <t>Move the event bus off in-process</t>
-        </is>
-      </c>
-      <c r="D14" s="10" t="inlineStr">
-        <is>
-          <t>Done</t>
+          <t>Tune SLA_TIER_SKIP_PENALTY values</t>
+        </is>
+      </c>
+      <c r="D14" s="5" t="inlineStr">
+        <is>
+          <t>Open</t>
         </is>
       </c>
       <c r="E14" s="6" t="inlineStr">
         <is>
-          <t>Phase 5</t>
+          <t>Phase 4 / I5</t>
         </is>
       </c>
       <c r="F14" s="6" t="inlineStr">
         <is>
-          <t>As the platform running on more than one instance, I want the event bus backed by Redis instead of in-process memory, so that hold-release and dispatch events stay consistent across multiple app instances.</t>
+          <t>As a hub dispatcher, I want the SLA tier skip penalties tuned to real route economics, so that the optimizer's tier prioritization reflects actual cost tradeoffs instead of a placeholder ordering.</t>
         </is>
       </c>
     </row>
     <row r="15">
       <c r="A15" s="7" t="inlineStr">
         <is>
-          <t>E9</t>
+          <t>E3</t>
         </is>
       </c>
       <c r="B15" s="8" t="inlineStr">
@@ -1092,7 +1092,7 @@
       </c>
       <c r="C15" s="8" t="inlineStr">
         <is>
-          <t>Validate the 2.5 DPH figure</t>
+          <t>Confirm real Epicor payload field names</t>
         </is>
       </c>
       <c r="D15" s="7" t="inlineStr">
@@ -1102,19 +1102,19 @@
       </c>
       <c r="E15" s="8" t="inlineStr">
         <is>
-          <t>Phase 9 (needs B2)</t>
+          <t>Phase 4 (needs B2)</t>
         </is>
       </c>
       <c r="F15" s="8" t="inlineStr">
         <is>
-          <t>As LMX leadership, I want the 2.5 deliveries-per-hour assumption validated against real Hub 1 data, so that pricing and staffing decisions rest on a proven number instead of a model assumption.</t>
+          <t>As the engineer integrating with a client's Epicor system, I want the real payload field names confirmed against a live tenant, so that orders ingest correctly instead of failing on a guessed schema.</t>
         </is>
       </c>
     </row>
     <row r="16">
       <c r="A16" s="5" t="inlineStr">
         <is>
-          <t>E10</t>
+          <t>E4</t>
         </is>
       </c>
       <c r="B16" s="6" t="inlineStr">
@@ -1124,7 +1124,7 @@
       </c>
       <c r="C16" s="6" t="inlineStr">
         <is>
-          <t>Tune HOT_SHOT's skip-penalty/hold-window placeholders</t>
+          <t>Verify the batch-hold 4-question decision logic</t>
         </is>
       </c>
       <c r="D16" s="5" t="inlineStr">
@@ -1134,61 +1134,61 @@
       </c>
       <c r="E16" s="6" t="inlineStr">
         <is>
-          <t>Phase 8 follow-up / I5</t>
+          <t>Phase 4 (needs B3)</t>
         </is>
       </c>
       <c r="F16" s="6" t="inlineStr">
         <is>
-          <t>As a hub dispatcher, I want HOT_SHOT's skip-penalty and hold-window values calibrated like the other tiers, so that the premium tier's priority handling is based on real economics, not a guess.</t>
+          <t>As a hub dispatcher, I want the batch-hold decision logic verified against the canonical spec, so that commingling decisions match the intended design rather than a reconstructed interpretation.</t>
         </is>
       </c>
     </row>
     <row r="17">
       <c r="A17" s="7" t="inlineStr">
         <is>
-          <t>S1</t>
+          <t>E5</t>
         </is>
       </c>
       <c r="B17" s="8" t="inlineStr">
         <is>
-          <t>Security</t>
+          <t>Core backend</t>
         </is>
       </c>
       <c r="C17" s="8" t="inlineStr">
         <is>
-          <t>Real per-user authentication for the ops dashboard</t>
-        </is>
-      </c>
-      <c r="D17" s="9" t="inlineStr">
-        <is>
-          <t>Done</t>
+          <t>Recalibrate SLA hold-window minutes</t>
+        </is>
+      </c>
+      <c r="D17" s="7" t="inlineStr">
+        <is>
+          <t>Open</t>
         </is>
       </c>
       <c r="E17" s="8" t="inlineStr">
         <is>
-          <t>Phase 5</t>
+          <t>Phase 4 / I5</t>
         </is>
       </c>
       <c r="F17" s="8" t="inlineStr">
         <is>
-          <t>As a hub ops manager, I want each staff member to log in with their own account and role, so that I know who did what in the dashboard and can limit admin actions to admins.</t>
+          <t>As a hub dispatcher, I want the SLA hold-window minutes recalibrated from real Hub 1 data, so that orders are held just long enough to batch efficiently without risking an SLA breach.</t>
         </is>
       </c>
     </row>
     <row r="18">
       <c r="A18" s="5" t="inlineStr">
         <is>
-          <t>S2</t>
+          <t>E6</t>
         </is>
       </c>
       <c r="B18" s="6" t="inlineStr">
         <is>
-          <t>Security</t>
+          <t>Core backend</t>
         </is>
       </c>
       <c r="C18" s="6" t="inlineStr">
         <is>
-          <t>Secrets management</t>
+          <t>Confirm Learning Loop flag-type naming convention</t>
         </is>
       </c>
       <c r="D18" s="5" t="inlineStr">
@@ -1198,66 +1198,66 @@
       </c>
       <c r="E18" s="6" t="inlineStr">
         <is>
-          <t>Phase 5</t>
+          <t>Phase 4</t>
         </is>
       </c>
       <c r="F18" s="6" t="inlineStr">
         <is>
-          <t>As the engineering team, I want credentials stored in a real secrets manager instead of a .env file, so that a leaked file or repo doesn't hand over database passwords and API keys.</t>
+          <t>As the engineer building the annotation loop, I want the flag-type naming convention signed off by a driver-app stakeholder, so that the contract between driver annotations and the Learning Loop isn't just an internal guess.</t>
         </is>
       </c>
     </row>
     <row r="19">
       <c r="A19" s="7" t="inlineStr">
         <is>
-          <t>S3</t>
+          <t>E7</t>
         </is>
       </c>
       <c r="B19" s="8" t="inlineStr">
         <is>
-          <t>Security</t>
+          <t>Core backend</t>
         </is>
       </c>
       <c r="C19" s="8" t="inlineStr">
         <is>
-          <t>A real production hosting decision</t>
-        </is>
-      </c>
-      <c r="D19" s="7" t="inlineStr">
-        <is>
-          <t>Open</t>
+          <t>Wire a real scheduler for the Learning Loop's nightly job</t>
+        </is>
+      </c>
+      <c r="D19" s="9" t="inlineStr">
+        <is>
+          <t>Done</t>
         </is>
       </c>
       <c r="E19" s="8" t="inlineStr">
         <is>
-          <t>Phase 5</t>
+          <t>Phase 4</t>
         </is>
       </c>
       <c r="F19" s="8" t="inlineStr">
         <is>
-          <t>As the engineering team preparing for Hub 1, I want a resilient hosting setup instead of a single-instance docker-compose, so that a container crash or server failure doesn't take down dispatch for real drivers and orders.</t>
+          <t>As a hub, I want the Learning Loop's nightly detection job to run automatically on schedule, so that rule proposals get generated every night without anyone manually triggering it.</t>
         </is>
       </c>
     </row>
     <row r="20">
       <c r="A20" s="5" t="inlineStr">
         <is>
-          <t>S4</t>
+          <t>E8</t>
         </is>
       </c>
       <c r="B20" s="6" t="inlineStr">
         <is>
-          <t>Security</t>
+          <t>Core backend</t>
         </is>
       </c>
       <c r="C20" s="6" t="inlineStr">
         <is>
-          <t>Observability</t>
-        </is>
-      </c>
-      <c r="D20" s="11" t="inlineStr">
-        <is>
-          <t>Partial</t>
+          <t>Move the event bus off in-process</t>
+        </is>
+      </c>
+      <c r="D20" s="10" t="inlineStr">
+        <is>
+          <t>Done</t>
         </is>
       </c>
       <c r="E20" s="6" t="inlineStr">
@@ -1267,56 +1267,56 @@
       </c>
       <c r="F20" s="6" t="inlineStr">
         <is>
-          <t>As an on-call engineer, I want error tracking and alerting layered on top of the existing metrics, so that I find out about a production problem from a page, not from a driver's phone call.</t>
+          <t>As the platform running on more than one instance, I want the event bus backed by Redis instead of in-process memory, so that hold-release and dispatch events stay consistent across multiple app instances.</t>
         </is>
       </c>
     </row>
     <row r="21">
       <c r="A21" s="7" t="inlineStr">
         <is>
-          <t>S5</t>
+          <t>E9</t>
         </is>
       </c>
       <c r="B21" s="8" t="inlineStr">
         <is>
-          <t>Security</t>
+          <t>Core backend</t>
         </is>
       </c>
       <c r="C21" s="8" t="inlineStr">
         <is>
-          <t>General API rate limiting</t>
-        </is>
-      </c>
-      <c r="D21" s="9" t="inlineStr">
-        <is>
-          <t>Done</t>
+          <t>Validate the 2.5 DPH figure</t>
+        </is>
+      </c>
+      <c r="D21" s="7" t="inlineStr">
+        <is>
+          <t>Open</t>
         </is>
       </c>
       <c r="E21" s="8" t="inlineStr">
         <is>
-          <t>Phase 5</t>
+          <t>Phase 9 (needs B2)</t>
         </is>
       </c>
       <c r="F21" s="8" t="inlineStr">
         <is>
-          <t>As the platform, I want a per-IP rate limit across the whole API, so that abusive traffic or credential-guessing can't overwhelm the system before authentication even runs.</t>
+          <t>As LMX leadership, I want the 2.5 deliveries-per-hour assumption validated against real Hub 1 data, so that pricing and staffing decisions rest on a proven number instead of a model assumption.</t>
         </is>
       </c>
     </row>
     <row r="22">
       <c r="A22" s="5" t="inlineStr">
         <is>
-          <t>S6</t>
+          <t>E10</t>
         </is>
       </c>
       <c r="B22" s="6" t="inlineStr">
         <is>
-          <t>Security</t>
+          <t>Core backend</t>
         </is>
       </c>
       <c r="C22" s="6" t="inlineStr">
         <is>
-          <t>A real security review</t>
+          <t>Tune HOT_SHOT's skip-penalty/hold-window placeholders</t>
         </is>
       </c>
       <c r="D22" s="5" t="inlineStr">
@@ -1326,19 +1326,19 @@
       </c>
       <c r="E22" s="6" t="inlineStr">
         <is>
-          <t>Phase 5</t>
+          <t>Phase 8 follow-up / I5</t>
         </is>
       </c>
       <c r="F22" s="6" t="inlineStr">
         <is>
-          <t>As LMX leadership, I want an outside security review of the platform, so that real orders, drivers, and eventually payments aren't the first real test of its defenses.</t>
+          <t>As a hub dispatcher, I want HOT_SHOT's skip-penalty and hold-window values calibrated like the other tiers, so that the premium tier's priority handling is based on real economics, not a guess.</t>
         </is>
       </c>
     </row>
     <row r="23">
       <c r="A23" s="7" t="inlineStr">
         <is>
-          <t>S7</t>
+          <t>S1</t>
         </is>
       </c>
       <c r="B23" s="8" t="inlineStr">
@@ -1348,7 +1348,7 @@
       </c>
       <c r="C23" s="8" t="inlineStr">
         <is>
-          <t>Twilio inbound-webhook signature verification</t>
+          <t>Real per-user authentication for the ops dashboard</t>
         </is>
       </c>
       <c r="D23" s="9" t="inlineStr">
@@ -1363,14 +1363,14 @@
       </c>
       <c r="F23" s="8" t="inlineStr">
         <is>
-          <t>As the platform receiving inbound SMS webhooks, I want Twilio's signature verified on every request, so that a forged webhook can't inject fake driver replies into the system.</t>
+          <t>As a hub ops manager, I want each staff member to log in with their own account and role, so that I know who did what in the dashboard and can limit admin actions to admins.</t>
         </is>
       </c>
     </row>
     <row r="24">
       <c r="A24" s="5" t="inlineStr">
         <is>
-          <t>S8</t>
+          <t>S2</t>
         </is>
       </c>
       <c r="B24" s="6" t="inlineStr">
@@ -1380,12 +1380,12 @@
       </c>
       <c r="C24" s="6" t="inlineStr">
         <is>
-          <t>Rate-limit client login</t>
-        </is>
-      </c>
-      <c r="D24" s="10" t="inlineStr">
-        <is>
-          <t>Done</t>
+          <t>Secrets management</t>
+        </is>
+      </c>
+      <c r="D24" s="5" t="inlineStr">
+        <is>
+          <t>Open</t>
         </is>
       </c>
       <c r="E24" s="6" t="inlineStr">
@@ -1395,14 +1395,14 @@
       </c>
       <c r="F24" s="6" t="inlineStr">
         <is>
-          <t>As a client company logging into the portal, I want login attempts rate-limited, so that someone else can't brute-force my company's portal password.</t>
+          <t>As the engineering team, I want credentials stored in a real secrets manager instead of a .env file, so that a leaked file or repo doesn't hand over database passwords and API keys.</t>
         </is>
       </c>
     </row>
     <row r="25">
       <c r="A25" s="7" t="inlineStr">
         <is>
-          <t>S9</t>
+          <t>S3</t>
         </is>
       </c>
       <c r="B25" s="8" t="inlineStr">
@@ -1412,12 +1412,12 @@
       </c>
       <c r="C25" s="8" t="inlineStr">
         <is>
-          <t>Enforce distinct client/driver JWT secrets at startup</t>
-        </is>
-      </c>
-      <c r="D25" s="9" t="inlineStr">
-        <is>
-          <t>Done</t>
+          <t>A real production hosting decision</t>
+        </is>
+      </c>
+      <c r="D25" s="7" t="inlineStr">
+        <is>
+          <t>Open</t>
         </is>
       </c>
       <c r="E25" s="8" t="inlineStr">
@@ -1427,56 +1427,56 @@
       </c>
       <c r="F25" s="8" t="inlineStr">
         <is>
-          <t>As the platform, I want the client and driver JWT secrets to be provably different at startup, so that a token issued for one audience can never be replayed as if it were the other.</t>
+          <t>As the engineering team preparing for Hub 1, I want a resilient hosting setup instead of a single-instance docker-compose, so that a container crash or server failure doesn't take down dispatch for real drivers and orders.</t>
         </is>
       </c>
     </row>
     <row r="26">
       <c r="A26" s="5" t="inlineStr">
         <is>
-          <t>D1</t>
+          <t>S4</t>
         </is>
       </c>
       <c r="B26" s="6" t="inlineStr">
         <is>
-          <t>Ops dashboard</t>
+          <t>Security</t>
         </is>
       </c>
       <c r="C26" s="6" t="inlineStr">
         <is>
-          <t>Add a list-hubs endpoint</t>
-        </is>
-      </c>
-      <c r="D26" s="10" t="inlineStr">
-        <is>
-          <t>Done</t>
+          <t>Observability</t>
+        </is>
+      </c>
+      <c r="D26" s="11" t="inlineStr">
+        <is>
+          <t>Partial</t>
         </is>
       </c>
       <c r="E26" s="6" t="inlineStr">
         <is>
-          <t>-</t>
+          <t>Phase 5</t>
         </is>
       </c>
       <c r="F26" s="6" t="inlineStr">
         <is>
-          <t>As a hub ops staff member, I want to pick my hub from a real dropdown instead of typing a UUID, so that I can't accidentally point the dashboard at the wrong hub.</t>
+          <t>As an on-call engineer, I want error tracking and alerting layered on top of the existing metrics, so that I find out about a production problem from a page, not from a driver's phone call.</t>
         </is>
       </c>
     </row>
     <row r="27">
       <c r="A27" s="7" t="inlineStr">
         <is>
-          <t>D2</t>
+          <t>S5</t>
         </is>
       </c>
       <c r="B27" s="8" t="inlineStr">
         <is>
-          <t>Ops dashboard</t>
+          <t>Security</t>
         </is>
       </c>
       <c r="C27" s="8" t="inlineStr">
         <is>
-          <t>Stop baking the API URL in at Docker build time</t>
+          <t>General API rate limiting</t>
         </is>
       </c>
       <c r="D27" s="9" t="inlineStr">
@@ -1486,29 +1486,29 @@
       </c>
       <c r="E27" s="8" t="inlineStr">
         <is>
-          <t>-</t>
+          <t>Phase 5</t>
         </is>
       </c>
       <c r="F27" s="8" t="inlineStr">
         <is>
-          <t>As the engineer deploying the dashboard, I want the API URL configured at container start instead of baked in at build time, so that one built image can point at any environment without a rebuild.</t>
+          <t>As the platform, I want a per-IP rate limit across the whole API, so that abusive traffic or credential-guessing can't overwhelm the system before authentication even runs.</t>
         </is>
       </c>
     </row>
     <row r="28">
       <c r="A28" s="5" t="inlineStr">
         <is>
-          <t>A1</t>
+          <t>S6</t>
         </is>
       </c>
       <c r="B28" s="6" t="inlineStr">
         <is>
-          <t>Driver app</t>
+          <t>Security</t>
         </is>
       </c>
       <c r="C28" s="6" t="inlineStr">
         <is>
-          <t>Push notifications</t>
+          <t>A real security review</t>
         </is>
       </c>
       <c r="D28" s="5" t="inlineStr">
@@ -1518,179 +1518,179 @@
       </c>
       <c r="E28" s="6" t="inlineStr">
         <is>
-          <t>Phase 6</t>
+          <t>Phase 5</t>
         </is>
       </c>
       <c r="F28" s="6" t="inlineStr">
         <is>
-          <t>As a driver, I want a push notification the moment a new job is offered to me, so that I don't have to keep the app open and polling to catch new work.</t>
+          <t>As LMX leadership, I want an outside security review of the platform, so that real orders, drivers, and eventually payments aren't the first real test of its defenses.</t>
         </is>
       </c>
     </row>
     <row r="29">
       <c r="A29" s="7" t="inlineStr">
         <is>
-          <t>A2</t>
+          <t>S7</t>
         </is>
       </c>
       <c r="B29" s="8" t="inlineStr">
         <is>
-          <t>Driver app</t>
+          <t>Security</t>
         </is>
       </c>
       <c r="C29" s="8" t="inlineStr">
         <is>
-          <t>Real camera/barcode scanning</t>
-        </is>
-      </c>
-      <c r="D29" s="7" t="inlineStr">
-        <is>
-          <t>Open</t>
+          <t>Twilio inbound-webhook signature verification</t>
+        </is>
+      </c>
+      <c r="D29" s="9" t="inlineStr">
+        <is>
+          <t>Done</t>
         </is>
       </c>
       <c r="E29" s="8" t="inlineStr">
         <is>
-          <t>Phase 6</t>
+          <t>Phase 5</t>
         </is>
       </c>
       <c r="F29" s="8" t="inlineStr">
         <is>
-          <t>As a driver scanning parcels at pickup, I want to scan a real barcode, so that the parcel count is accurate instead of a manual tap anyone could get wrong or fake.</t>
+          <t>As the platform receiving inbound SMS webhooks, I want Twilio's signature verified on every request, so that a forged webhook can't inject fake driver replies into the system.</t>
         </is>
       </c>
     </row>
     <row r="30">
       <c r="A30" s="5" t="inlineStr">
         <is>
-          <t>A3</t>
+          <t>S8</t>
         </is>
       </c>
       <c r="B30" s="6" t="inlineStr">
         <is>
-          <t>Driver app</t>
+          <t>Security</t>
         </is>
       </c>
       <c r="C30" s="6" t="inlineStr">
         <is>
-          <t>Real photo/signature capture + upload pipeline</t>
-        </is>
-      </c>
-      <c r="D30" s="5" t="inlineStr">
-        <is>
-          <t>Open</t>
+          <t>Rate-limit client login</t>
+        </is>
+      </c>
+      <c r="D30" s="10" t="inlineStr">
+        <is>
+          <t>Done</t>
         </is>
       </c>
       <c r="E30" s="6" t="inlineStr">
         <is>
-          <t>Phase 6</t>
+          <t>Phase 5</t>
         </is>
       </c>
       <c r="F30" s="6" t="inlineStr">
         <is>
-          <t>As a driver completing a delivery, I want to actually capture and upload a photo or signature, so that proof of delivery is a real image on file, not a placeholder URL.</t>
+          <t>As a client company logging into the portal, I want login attempts rate-limited, so that someone else can't brute-force my company's portal password.</t>
         </is>
       </c>
     </row>
     <row r="31">
       <c r="A31" s="7" t="inlineStr">
         <is>
-          <t>A4</t>
+          <t>S9</t>
         </is>
       </c>
       <c r="B31" s="8" t="inlineStr">
         <is>
-          <t>Driver app</t>
+          <t>Security</t>
         </is>
       </c>
       <c r="C31" s="8" t="inlineStr">
         <is>
-          <t>A real PIN-issuance/verification system</t>
-        </is>
-      </c>
-      <c r="D31" s="7" t="inlineStr">
-        <is>
-          <t>Open</t>
+          <t>Enforce distinct client/driver JWT secrets at startup</t>
+        </is>
+      </c>
+      <c r="D31" s="9" t="inlineStr">
+        <is>
+          <t>Done</t>
         </is>
       </c>
       <c r="E31" s="8" t="inlineStr">
         <is>
-          <t>Phase 6</t>
+          <t>Phase 5</t>
         </is>
       </c>
       <c r="F31" s="8" t="inlineStr">
         <is>
-          <t>As a driver delivering an order that requires a PIN, I want the PIN checked against a real system, so that I can be confident the person receiving the package is who they say they are.</t>
+          <t>As the platform, I want the client and driver JWT secrets to be provably different at startup, so that a token issued for one audience can never be replayed as if it were the other.</t>
         </is>
       </c>
     </row>
     <row r="32">
       <c r="A32" s="5" t="inlineStr">
         <is>
-          <t>A5</t>
+          <t>D1</t>
         </is>
       </c>
       <c r="B32" s="6" t="inlineStr">
         <is>
-          <t>Driver app</t>
+          <t>Ops dashboard</t>
         </is>
       </c>
       <c r="C32" s="6" t="inlineStr">
         <is>
-          <t>Maps SDK / turn-by-turn navigation</t>
-        </is>
-      </c>
-      <c r="D32" s="5" t="inlineStr">
-        <is>
-          <t>Open</t>
+          <t>Add a list-hubs endpoint</t>
+        </is>
+      </c>
+      <c r="D32" s="10" t="inlineStr">
+        <is>
+          <t>Done</t>
         </is>
       </c>
       <c r="E32" s="6" t="inlineStr">
         <is>
-          <t>Phase 6</t>
+          <t>-</t>
         </is>
       </c>
       <c r="F32" s="6" t="inlineStr">
         <is>
-          <t>As a driver on route, I want live turn-by-turn navigation in the app, so that I don't need a separate maps app to find each stop.</t>
+          <t>As a hub ops staff member, I want to pick my hub from a real dropdown instead of typing a UUID, so that I can't accidentally point the dashboard at the wrong hub.</t>
         </is>
       </c>
     </row>
     <row r="33">
       <c r="A33" s="7" t="inlineStr">
         <is>
-          <t>A6</t>
+          <t>D2</t>
         </is>
       </c>
       <c r="B33" s="8" t="inlineStr">
         <is>
-          <t>Driver app</t>
+          <t>Ops dashboard</t>
         </is>
       </c>
       <c r="C33" s="8" t="inlineStr">
         <is>
-          <t>Mobile app store deployment pipeline</t>
-        </is>
-      </c>
-      <c r="D33" s="7" t="inlineStr">
-        <is>
-          <t>Open</t>
+          <t>Stop baking the API URL in at Docker build time</t>
+        </is>
+      </c>
+      <c r="D33" s="9" t="inlineStr">
+        <is>
+          <t>Done</t>
         </is>
       </c>
       <c r="E33" s="8" t="inlineStr">
         <is>
-          <t>Phase 6</t>
+          <t>-</t>
         </is>
       </c>
       <c r="F33" s="8" t="inlineStr">
         <is>
-          <t>As a driver, I want to install the app from TestFlight or the Play Store, so that I don't need developer tooling just to get the app on my phone.</t>
+          <t>As the engineer deploying the dashboard, I want the API URL configured at container start instead of baked in at build time, so that one built image can point at any environment without a rebuild.</t>
         </is>
       </c>
     </row>
     <row r="34">
       <c r="A34" s="5" t="inlineStr">
         <is>
-          <t>A7</t>
+          <t>A1</t>
         </is>
       </c>
       <c r="B34" s="6" t="inlineStr">
@@ -1700,7 +1700,7 @@
       </c>
       <c r="C34" s="6" t="inlineStr">
         <is>
-          <t>Masked voice calling</t>
+          <t>Push notifications</t>
         </is>
       </c>
       <c r="D34" s="5" t="inlineStr">
@@ -1715,14 +1715,14 @@
       </c>
       <c r="F34" s="6" t="inlineStr">
         <is>
-          <t>As a driver or customer who needs to talk instead of text, I want a masked voice call option, so that we can resolve an issue quickly without exposing either party's real phone number.</t>
+          <t>As a driver, I want a push notification the moment a new job is offered to me, so that I don't have to keep the app open and polling to catch new work.</t>
         </is>
       </c>
     </row>
     <row r="35">
       <c r="A35" s="7" t="inlineStr">
         <is>
-          <t>A8</t>
+          <t>A2</t>
         </is>
       </c>
       <c r="B35" s="8" t="inlineStr">
@@ -1732,12 +1732,12 @@
       </c>
       <c r="C35" s="8" t="inlineStr">
         <is>
-          <t>Harden inbound-SMS reply matching</t>
-        </is>
-      </c>
-      <c r="D35" s="9" t="inlineStr">
-        <is>
-          <t>Done</t>
+          <t>Real camera/barcode scanning</t>
+        </is>
+      </c>
+      <c r="D35" s="7" t="inlineStr">
+        <is>
+          <t>Open</t>
         </is>
       </c>
       <c r="E35" s="8" t="inlineStr">
@@ -1747,14 +1747,14 @@
       </c>
       <c r="F35" s="8" t="inlineStr">
         <is>
-          <t>As a shop replying to a delivery SMS, I want my reply matched to the correct, active conversation, so that my message doesn't get attached to the wrong or already-completed stop.</t>
+          <t>As a driver scanning parcels at pickup, I want to scan a real barcode, so that the parcel count is accurate instead of a manual tap anyone could get wrong or fake.</t>
         </is>
       </c>
     </row>
     <row r="36">
       <c r="A36" s="5" t="inlineStr">
         <is>
-          <t>A9</t>
+          <t>A3</t>
         </is>
       </c>
       <c r="B36" s="6" t="inlineStr">
@@ -1764,381 +1764,381 @@
       </c>
       <c r="C36" s="6" t="inlineStr">
         <is>
-          <t>Real earnings formula + payroll integration</t>
-        </is>
-      </c>
-      <c r="D36" s="11" t="inlineStr">
-        <is>
-          <t>Partial (scaffolding shipped)</t>
+          <t>Real photo/signature capture + upload pipeline</t>
+        </is>
+      </c>
+      <c r="D36" s="5" t="inlineStr">
+        <is>
+          <t>Open</t>
         </is>
       </c>
       <c r="E36" s="6" t="inlineStr">
         <is>
-          <t>Phase 7</t>
+          <t>Phase 6</t>
         </is>
       </c>
       <c r="F36" s="6" t="inlineStr">
         <is>
-          <t>As a driver, I want my earnings screen to show a real, calculated number tied to actual payroll, so that I know what I'll actually be paid instead of seeing a placeholder.</t>
+          <t>As a driver completing a delivery, I want to actually capture and upload a photo or signature, so that proof of delivery is a real image on file, not a placeholder URL.</t>
         </is>
       </c>
     </row>
     <row r="37">
       <c r="A37" s="7" t="inlineStr">
         <is>
-          <t>C1</t>
+          <t>A4</t>
         </is>
       </c>
       <c r="B37" s="8" t="inlineStr">
         <is>
-          <t>Components</t>
+          <t>Driver app</t>
         </is>
       </c>
       <c r="C37" s="8" t="inlineStr">
         <is>
-          <t>Client-facing dashboard</t>
-        </is>
-      </c>
-      <c r="D37" s="9" t="inlineStr">
-        <is>
-          <t>Done (Phase 8)</t>
+          <t>A real PIN-issuance/verification system</t>
+        </is>
+      </c>
+      <c r="D37" s="7" t="inlineStr">
+        <is>
+          <t>Open</t>
         </is>
       </c>
       <c r="E37" s="8" t="inlineStr">
         <is>
-          <t>-</t>
+          <t>Phase 6</t>
         </is>
       </c>
       <c r="F37" s="8" t="inlineStr">
         <is>
-          <t>As a client company, I want a portal showing my order history, status, and fees, so that I don't have to call LMX to know where my orders stand.</t>
+          <t>As a driver delivering an order that requires a PIN, I want the PIN checked against a real system, so that I can be confident the person receiving the package is who they say they are.</t>
         </is>
       </c>
     </row>
     <row r="38">
       <c r="A38" s="5" t="inlineStr">
         <is>
-          <t>C2</t>
+          <t>A5</t>
         </is>
       </c>
       <c r="B38" s="6" t="inlineStr">
         <is>
-          <t>Components</t>
+          <t>Driver app</t>
         </is>
       </c>
       <c r="C38" s="6" t="inlineStr">
         <is>
-          <t>Shop SMS</t>
-        </is>
-      </c>
-      <c r="D38" s="10" t="inlineStr">
-        <is>
-          <t>Done (Phase 8)</t>
+          <t>Maps SDK / turn-by-turn navigation</t>
+        </is>
+      </c>
+      <c r="D38" s="5" t="inlineStr">
+        <is>
+          <t>Open</t>
         </is>
       </c>
       <c r="E38" s="6" t="inlineStr">
         <is>
-          <t>-</t>
+          <t>Phase 6</t>
         </is>
       </c>
       <c r="F38" s="6" t="inlineStr">
         <is>
-          <t>As a shop, I want an automatic text when my order is picked up and when the driver's en route, so that I don't have to guess or call in to check.</t>
+          <t>As a driver on route, I want live turn-by-turn navigation in the app, so that I don't need a separate maps app to find each stop.</t>
         </is>
       </c>
     </row>
     <row r="39">
       <c r="A39" s="7" t="inlineStr">
         <is>
-          <t>C3</t>
+          <t>A6</t>
         </is>
       </c>
       <c r="B39" s="8" t="inlineStr">
         <is>
-          <t>Components</t>
+          <t>Driver app</t>
         </is>
       </c>
       <c r="C39" s="8" t="inlineStr">
         <is>
-          <t>A real billing/invoicing system</t>
-        </is>
-      </c>
-      <c r="D39" s="12" t="inlineStr">
-        <is>
-          <t>Partial</t>
+          <t>Mobile app store deployment pipeline</t>
+        </is>
+      </c>
+      <c r="D39" s="7" t="inlineStr">
+        <is>
+          <t>Open</t>
         </is>
       </c>
       <c r="E39" s="8" t="inlineStr">
         <is>
-          <t>Phase 8 follow-up</t>
+          <t>Phase 6</t>
         </is>
       </c>
       <c r="F39" s="8" t="inlineStr">
         <is>
-          <t>As a client company, I want a real monthly statement and invoice I can download, so that I can reconcile what I owe LMX without manually recomputing it from order history.</t>
+          <t>As a driver, I want to install the app from TestFlight or the Play Store, so that I don't need developer tooling just to get the app on my phone.</t>
         </is>
       </c>
     </row>
     <row r="40">
       <c r="A40" s="5" t="inlineStr">
         <is>
-          <t>C4</t>
+          <t>A7</t>
         </is>
       </c>
       <c r="B40" s="6" t="inlineStr">
         <is>
-          <t>Components</t>
+          <t>Driver app</t>
         </is>
       </c>
       <c r="C40" s="6" t="inlineStr">
         <is>
-          <t>Multi-user client accounts</t>
+          <t>Masked voice calling</t>
         </is>
       </c>
       <c r="D40" s="5" t="inlineStr">
         <is>
-          <t>Open (deliberate, later)</t>
+          <t>Open</t>
         </is>
       </c>
       <c r="E40" s="6" t="inlineStr">
         <is>
-          <t>Phase 8 follow-up</t>
+          <t>Phase 6</t>
         </is>
       </c>
       <c r="F40" s="6" t="inlineStr">
         <is>
-          <t>As a client company with both an AP contact and an ops contact, I want more than one login for my company, so that each person can access the portal without sharing one password.</t>
+          <t>As a driver or customer who needs to talk instead of text, I want a masked voice call option, so that we can resolve an issue quickly without exposing either party's real phone number.</t>
         </is>
       </c>
     </row>
     <row r="41">
       <c r="A41" s="7" t="inlineStr">
         <is>
-          <t>C5</t>
+          <t>A8</t>
         </is>
       </c>
       <c r="B41" s="8" t="inlineStr">
         <is>
-          <t>Components</t>
+          <t>Driver app</t>
         </is>
       </c>
       <c r="C41" s="8" t="inlineStr">
         <is>
-          <t>Self-service client signup</t>
-        </is>
-      </c>
-      <c r="D41" s="13" t="inlineStr">
-        <is>
-          <t>Deliberately not building</t>
+          <t>Harden inbound-SMS reply matching</t>
+        </is>
+      </c>
+      <c r="D41" s="9" t="inlineStr">
+        <is>
+          <t>Done</t>
         </is>
       </c>
       <c r="E41" s="8" t="inlineStr">
         <is>
-          <t>-</t>
+          <t>Phase 6</t>
         </is>
       </c>
       <c r="F41" s="8" t="inlineStr">
         <is>
-          <t>As LMX's business development team, we deliberately do not want a self-serve client signup flow, so that every new client relationship stays a real onboarding conversation, matching a B2B operator model rather than self-serve SaaS.</t>
+          <t>As a shop replying to a delivery SMS, I want my reply matched to the correct, active conversation, so that my message doesn't get attached to the wrong or already-completed stop.</t>
         </is>
       </c>
     </row>
     <row r="42">
       <c r="A42" s="5" t="inlineStr">
         <is>
-          <t>P1</t>
+          <t>A9</t>
         </is>
       </c>
       <c r="B42" s="6" t="inlineStr">
         <is>
-          <t>Autonomy partners</t>
+          <t>Driver app</t>
         </is>
       </c>
       <c r="C42" s="6" t="inlineStr">
         <is>
-          <t>Courier abstraction over the fleet model</t>
-        </is>
-      </c>
-      <c r="D42" s="5" t="inlineStr">
-        <is>
-          <t>Open</t>
+          <t>Real earnings formula + payroll integration</t>
+        </is>
+      </c>
+      <c r="D42" s="11" t="inlineStr">
+        <is>
+          <t>Partial (scaffolding shipped)</t>
         </is>
       </c>
       <c r="E42" s="6" t="inlineStr">
         <is>
-          <t>Phase 11 (Track A gate)</t>
+          <t>Phase 7</t>
         </is>
       </c>
       <c r="F42" s="6" t="inlineStr">
         <is>
-          <t>As the engineering team, I want the fleet model generalized into a courier abstraction (human driver, autonomy partner, or gig courier), so that adding a new capacity type later doesn't require reworking code that assumes every courier is a person.</t>
+          <t>As a driver, I want my earnings screen to show a real, calculated number tied to actual payroll, so that I know what I'll actually be paid instead of seeing a placeholder.</t>
         </is>
       </c>
     </row>
     <row r="43">
       <c r="A43" s="7" t="inlineStr">
         <is>
-          <t>P2</t>
+          <t>C1</t>
         </is>
       </c>
       <c r="B43" s="8" t="inlineStr">
         <is>
-          <t>Autonomy partners</t>
+          <t>Components</t>
         </is>
       </c>
       <c r="C43" s="8" t="inlineStr">
         <is>
-          <t>Capacity-provider adapter layer</t>
-        </is>
-      </c>
-      <c r="D43" s="7" t="inlineStr">
-        <is>
-          <t>Open</t>
+          <t>Client-facing dashboard</t>
+        </is>
+      </c>
+      <c r="D43" s="9" t="inlineStr">
+        <is>
+          <t>Done (Phase 8)</t>
         </is>
       </c>
       <c r="E43" s="8" t="inlineStr">
         <is>
-          <t>Phase 11 (Track A gate)</t>
+          <t>-</t>
         </is>
       </c>
       <c r="F43" s="8" t="inlineStr">
         <is>
-          <t>As the engineering team, I want one adapter per capacity partner normalizing capacity, assignment, and status, so that onboarding a new autonomy or gig partner doesn't mean writing bespoke dispatch logic each time.</t>
+          <t>As a client company, I want a portal showing my order history, status, and fees, so that I don't have to call LMX to know where my orders stand.</t>
         </is>
       </c>
     </row>
     <row r="44">
       <c r="A44" s="5" t="inlineStr">
         <is>
-          <t>P3</t>
+          <t>C2</t>
         </is>
       </c>
       <c r="B44" s="6" t="inlineStr">
         <is>
-          <t>Autonomy partners</t>
+          <t>Components</t>
         </is>
       </c>
       <c r="C44" s="6" t="inlineStr">
         <is>
-          <t>Mode-aware dispatch</t>
-        </is>
-      </c>
-      <c r="D44" s="5" t="inlineStr">
-        <is>
-          <t>Open</t>
+          <t>Shop SMS</t>
+        </is>
+      </c>
+      <c r="D44" s="10" t="inlineStr">
+        <is>
+          <t>Done (Phase 8)</t>
         </is>
       </c>
       <c r="E44" s="6" t="inlineStr">
         <is>
-          <t>Phase 11</t>
+          <t>-</t>
         </is>
       </c>
       <c r="F44" s="6" t="inlineStr">
         <is>
-          <t>As a hub dispatcher, I want the optimizer to filter and choose the cheapest eligible delivery mode per order, so that a 40lb order never gets offered to a bike courier and cost-per-drop stays optimized across every available mode.</t>
+          <t>As a shop, I want an automatic text when my order is picked up and when the driver's en route, so that I don't have to guess or call in to check.</t>
         </is>
       </c>
     </row>
     <row r="45">
       <c r="A45" s="7" t="inlineStr">
         <is>
-          <t>P4</t>
+          <t>C3</t>
         </is>
       </c>
       <c r="B45" s="8" t="inlineStr">
         <is>
-          <t>Autonomy partners</t>
+          <t>Components</t>
         </is>
       </c>
       <c r="C45" s="8" t="inlineStr">
         <is>
-          <t>Unmanned handoff + proof of delivery</t>
-        </is>
-      </c>
-      <c r="D45" s="7" t="inlineStr">
-        <is>
-          <t>Open</t>
+          <t>A real billing/invoicing system</t>
+        </is>
+      </c>
+      <c r="D45" s="12" t="inlineStr">
+        <is>
+          <t>Partial</t>
         </is>
       </c>
       <c r="E45" s="8" t="inlineStr">
         <is>
-          <t>Phase 11 (shares A4)</t>
+          <t>Phase 8 follow-up</t>
         </is>
       </c>
       <c r="F45" s="8" t="inlineStr">
         <is>
-          <t>As a shop receiving an autonomous vehicle for pickup, I want a clear load-confirmation flow, so that handing off a parcel to a bot is as unambiguous as handing it to a driver.</t>
+          <t>As a client company, I want a real monthly statement and invoice I can download, so that I can reconcile what I owe LMX without manually recomputing it from order history.</t>
         </is>
       </c>
     </row>
     <row r="46">
       <c r="A46" s="5" t="inlineStr">
         <is>
-          <t>P5</t>
+          <t>C4</t>
         </is>
       </c>
       <c r="B46" s="6" t="inlineStr">
         <is>
-          <t>Autonomy partners</t>
+          <t>Components</t>
         </is>
       </c>
       <c r="C46" s="6" t="inlineStr">
         <is>
-          <t>Partner settlement</t>
+          <t>Multi-user client accounts</t>
         </is>
       </c>
       <c r="D46" s="5" t="inlineStr">
         <is>
-          <t>Open</t>
+          <t>Open (deliberate, later)</t>
         </is>
       </c>
       <c r="E46" s="6" t="inlineStr">
         <is>
-          <t>Phase 11 (later)</t>
+          <t>Phase 8 follow-up</t>
         </is>
       </c>
       <c r="F46" s="6" t="inlineStr">
         <is>
-          <t>As an autonomy or gig-courier partner, I want a monthly settlement statement for the deliveries I carried, so that I get paid accurately without a manual reconciliation with LMX.</t>
+          <t>As a client company with both an AP contact and an ops contact, I want more than one login for my company, so that each person can access the portal without sharing one password.</t>
         </is>
       </c>
     </row>
     <row r="47">
       <c r="A47" s="7" t="inlineStr">
         <is>
-          <t>P6</t>
+          <t>C5</t>
         </is>
       </c>
       <c r="B47" s="8" t="inlineStr">
         <is>
-          <t>Autonomy partners</t>
+          <t>Components</t>
         </is>
       </c>
       <c r="C47" s="8" t="inlineStr">
         <is>
-          <t>Partner portal</t>
-        </is>
-      </c>
-      <c r="D47" s="7" t="inlineStr">
-        <is>
-          <t>Open</t>
+          <t>Self-service client signup</t>
+        </is>
+      </c>
+      <c r="D47" s="13" t="inlineStr">
+        <is>
+          <t>Deliberately not building</t>
         </is>
       </c>
       <c r="E47" s="8" t="inlineStr">
         <is>
-          <t>Phase 11 (later)</t>
+          <t>-</t>
         </is>
       </c>
       <c r="F47" s="8" t="inlineStr">
         <is>
-          <t>As an autonomy or gig-courier partner, I want a portal showing my delivery history and settlement statements, so that I can check my own performance and pay without emailing LMX ops.</t>
+          <t>As LMX's business development team, we deliberately do not want a self-serve client signup flow, so that every new client relationship stays a real onboarding conversation, matching a B2B operator model rather than self-serve SaaS.</t>
         </is>
       </c>
     </row>
     <row r="48">
       <c r="A48" s="5" t="inlineStr">
         <is>
-          <t>P7</t>
+          <t>P1</t>
         </is>
       </c>
       <c r="B48" s="6" t="inlineStr">
@@ -2148,39 +2148,39 @@
       </c>
       <c r="C48" s="6" t="inlineStr">
         <is>
-          <t>Gig-courier cost-optimized dispatch</t>
+          <t>Courier abstraction over the fleet model</t>
         </is>
       </c>
       <c r="D48" s="5" t="inlineStr">
         <is>
-          <t>Open (gated on unit economics)</t>
+          <t>Open</t>
         </is>
       </c>
       <c r="E48" s="6" t="inlineStr">
         <is>
-          <t>Phase 11 (Track B)</t>
+          <t>Phase 11 (Track A gate)</t>
         </is>
       </c>
       <c r="F48" s="6" t="inlineStr">
         <is>
-          <t>As LMX leadership, I want the option to route an order to a gig courier when it's genuinely the cheaper eligible choice, so that capacity can flex without ever changing the client's brand, SLA, or bill - capped and tagged so it never masks LMX's own unit economics.</t>
+          <t>As the engineering team, I want the fleet model generalized into a courier abstraction (human driver, autonomy partner, or gig courier), so that adding a new capacity type later doesn't require reworking code that assumes every courier is a person.</t>
         </is>
       </c>
     </row>
     <row r="49">
       <c r="A49" s="7" t="inlineStr">
         <is>
-          <t>F1</t>
+          <t>P2</t>
         </is>
       </c>
       <c r="B49" s="8" t="inlineStr">
         <is>
-          <t>Competitive gaps</t>
+          <t>Autonomy partners</t>
         </is>
       </c>
       <c r="C49" s="8" t="inlineStr">
         <is>
-          <t>Live driver location pipeline</t>
+          <t>Capacity-provider adapter layer</t>
         </is>
       </c>
       <c r="D49" s="7" t="inlineStr">
@@ -2190,29 +2190,29 @@
       </c>
       <c r="E49" s="8" t="inlineStr">
         <is>
-          <t>Phase 6</t>
+          <t>Phase 11 (Track A gate)</t>
         </is>
       </c>
       <c r="F49" s="8" t="inlineStr">
         <is>
-          <t>As the platform, I want the driver app to periodically report its location, so that there's a real, current position on file for every driver on shift.</t>
+          <t>As the engineering team, I want one adapter per capacity partner normalizing capacity, assignment, and status, so that onboarding a new autonomy or gig partner doesn't mean writing bespoke dispatch logic each time.</t>
         </is>
       </c>
     </row>
     <row r="50">
       <c r="A50" s="5" t="inlineStr">
         <is>
-          <t>F2</t>
+          <t>P3</t>
         </is>
       </c>
       <c r="B50" s="6" t="inlineStr">
         <is>
-          <t>Competitive gaps</t>
+          <t>Autonomy partners</t>
         </is>
       </c>
       <c r="C50" s="6" t="inlineStr">
         <is>
-          <t>Live map view (ops dashboard)</t>
+          <t>Mode-aware dispatch</t>
         </is>
       </c>
       <c r="D50" s="5" t="inlineStr">
@@ -2222,29 +2222,29 @@
       </c>
       <c r="E50" s="6" t="inlineStr">
         <is>
-          <t>Phase 6</t>
+          <t>Phase 11</t>
         </is>
       </c>
       <c r="F50" s="6" t="inlineStr">
         <is>
-          <t>As a hub ops manager, I want to see every driver's live position on a map, so that I know where my fleet actually is, not just what stop list each driver was assigned.</t>
+          <t>As a hub dispatcher, I want the optimizer to filter and choose the cheapest eligible delivery mode per order, so that a 40lb order never gets offered to a bike courier and cost-per-drop stays optimized across every available mode.</t>
         </is>
       </c>
     </row>
     <row r="51">
       <c r="A51" s="7" t="inlineStr">
         <is>
-          <t>F3</t>
+          <t>P4</t>
         </is>
       </c>
       <c r="B51" s="8" t="inlineStr">
         <is>
-          <t>Competitive gaps</t>
+          <t>Autonomy partners</t>
         </is>
       </c>
       <c r="C51" s="8" t="inlineStr">
         <is>
-          <t>Customer-facing live tracking page</t>
+          <t>Unmanned handoff + proof of delivery</t>
         </is>
       </c>
       <c r="D51" s="7" t="inlineStr">
@@ -2254,29 +2254,29 @@
       </c>
       <c r="E51" s="8" t="inlineStr">
         <is>
-          <t>Phase 8 follow-up</t>
+          <t>Phase 11 (shares A4)</t>
         </is>
       </c>
       <c r="F51" s="8" t="inlineStr">
         <is>
-          <t>As the person receiving a delivery, I want a link that shows my driver's live position and ETA, so that I don't have to call the shop or guess when my part will arrive.</t>
+          <t>As a shop receiving an autonomous vehicle for pickup, I want a clear load-confirmation flow, so that handing off a parcel to a bot is as unambiguous as handing it to a driver.</t>
         </is>
       </c>
     </row>
     <row r="52">
       <c r="A52" s="5" t="inlineStr">
         <is>
-          <t>F4</t>
+          <t>P5</t>
         </is>
       </c>
       <c r="B52" s="6" t="inlineStr">
         <is>
-          <t>Competitive gaps</t>
+          <t>Autonomy partners</t>
         </is>
       </c>
       <c r="C52" s="6" t="inlineStr">
         <is>
-          <t>Outbound status webhooks + integrations surface</t>
+          <t>Partner settlement</t>
         </is>
       </c>
       <c r="D52" s="5" t="inlineStr">
@@ -2286,29 +2286,29 @@
       </c>
       <c r="E52" s="6" t="inlineStr">
         <is>
-          <t>Phase 8 follow-up</t>
+          <t>Phase 11 (later)</t>
         </is>
       </c>
       <c r="F52" s="6" t="inlineStr">
         <is>
-          <t>As a client's system administrator, I want to subscribe to order status webhooks, so that my own systems update automatically instead of polling or waiting on a manual check.</t>
+          <t>As an autonomy or gig-courier partner, I want a monthly settlement statement for the deliveries I carried, so that I get paid accurately without a manual reconciliation with LMX.</t>
         </is>
       </c>
     </row>
     <row r="53">
       <c r="A53" s="7" t="inlineStr">
         <is>
-          <t>F5</t>
+          <t>P6</t>
         </is>
       </c>
       <c r="B53" s="8" t="inlineStr">
         <is>
-          <t>Competitive gaps</t>
+          <t>Autonomy partners</t>
         </is>
       </c>
       <c r="C53" s="8" t="inlineStr">
         <is>
-          <t>Flexible/rate-table billing</t>
+          <t>Partner portal</t>
         </is>
       </c>
       <c r="D53" s="7" t="inlineStr">
@@ -2318,51 +2318,51 @@
       </c>
       <c r="E53" s="8" t="inlineStr">
         <is>
-          <t>Phase 8 follow-up</t>
+          <t>Phase 11 (later)</t>
         </is>
       </c>
       <c r="F53" s="8" t="inlineStr">
         <is>
-          <t>As a client with orders of very different sizes, I want billing that can reflect piece count, weight, or mileage, not just a flat per-drop rate, so that pricing matches the actual cost of serving my orders.</t>
+          <t>As an autonomy or gig-courier partner, I want a portal showing my delivery history and settlement statements, so that I can check my own performance and pay without emailing LMX ops.</t>
         </is>
       </c>
     </row>
     <row r="54">
       <c r="A54" s="5" t="inlineStr">
         <is>
-          <t>F6</t>
+          <t>P7</t>
         </is>
       </c>
       <c r="B54" s="6" t="inlineStr">
         <is>
-          <t>Competitive gaps</t>
+          <t>Autonomy partners</t>
         </is>
       </c>
       <c r="C54" s="6" t="inlineStr">
         <is>
-          <t>Real-time mid-route re-optimization</t>
+          <t>Gig-courier cost-optimized dispatch</t>
         </is>
       </c>
       <c r="D54" s="5" t="inlineStr">
         <is>
-          <t>Open</t>
+          <t>Open (gated on unit economics)</t>
         </is>
       </c>
       <c r="E54" s="6" t="inlineStr">
         <is>
-          <t>Phase 4 (needs E1)</t>
+          <t>Phase 11 (Track B)</t>
         </is>
       </c>
       <c r="F54" s="6" t="inlineStr">
         <is>
-          <t>As a hub dispatcher, I want the optimizer to re-sequence an in-progress route when conditions change, so that a driver isn't stuck following a plan that's gone stale since the last cycle.</t>
+          <t>As LMX leadership, I want the option to route an order to a gig courier when it's genuinely the cheaper eligible choice, so that capacity can flex without ever changing the client's brand, SLA, or bill - capped and tagged so it never masks LMX's own unit economics.</t>
         </is>
       </c>
     </row>
     <row r="55">
       <c r="A55" s="7" t="inlineStr">
         <is>
-          <t>F7</t>
+          <t>F1</t>
         </is>
       </c>
       <c r="B55" s="8" t="inlineStr">
@@ -2372,7 +2372,7 @@
       </c>
       <c r="C55" s="8" t="inlineStr">
         <is>
-          <t>Client- and ops-facing analytics dashboards</t>
+          <t>Live driver location pipeline</t>
         </is>
       </c>
       <c r="D55" s="7" t="inlineStr">
@@ -2382,19 +2382,19 @@
       </c>
       <c r="E55" s="8" t="inlineStr">
         <is>
-          <t>Phase 10 (folds into I4)</t>
+          <t>Phase 6</t>
         </is>
       </c>
       <c r="F55" s="8" t="inlineStr">
         <is>
-          <t>As a client company, I want to see my own on-time rate, volume, and cost trend in the portal, so that I have concrete proof of the value of switching to per-drop pricing with LMX.</t>
+          <t>As the platform, I want the driver app to periodically report its location, so that there's a real, current position on file for every driver on shift.</t>
         </is>
       </c>
     </row>
     <row r="56">
       <c r="A56" s="5" t="inlineStr">
         <is>
-          <t>F8</t>
+          <t>F2</t>
         </is>
       </c>
       <c r="B56" s="6" t="inlineStr">
@@ -2404,7 +2404,7 @@
       </c>
       <c r="C56" s="6" t="inlineStr">
         <is>
-          <t>White-label / multi-brand portal theming</t>
+          <t>Live map view (ops dashboard)</t>
         </is>
       </c>
       <c r="D56" s="5" t="inlineStr">
@@ -2414,19 +2414,19 @@
       </c>
       <c r="E56" s="6" t="inlineStr">
         <is>
-          <t>Phase 8 follow-up</t>
+          <t>Phase 6</t>
         </is>
       </c>
       <c r="F56" s="6" t="inlineStr">
         <is>
-          <t>As a reselling partner, I want the client portal to carry my own brand, so that my customers experience it as part of my business, not a visibly third-party tool.</t>
+          <t>As a hub ops manager, I want to see every driver's live position on a map, so that I know where my fleet actually is, not just what stop list each driver was assigned.</t>
         </is>
       </c>
     </row>
     <row r="57">
       <c r="A57" s="7" t="inlineStr">
         <is>
-          <t>F9</t>
+          <t>F3</t>
         </is>
       </c>
       <c r="B57" s="8" t="inlineStr">
@@ -2436,29 +2436,29 @@
       </c>
       <c r="C57" s="8" t="inlineStr">
         <is>
-          <t>Hybrid gig-fleet overflow dispatch</t>
-        </is>
-      </c>
-      <c r="D57" s="13" t="inlineStr">
-        <is>
-          <t>Superseded -&gt; reinstated as P7</t>
+          <t>Customer-facing live tracking page</t>
+        </is>
+      </c>
+      <c r="D57" s="7" t="inlineStr">
+        <is>
+          <t>Open</t>
         </is>
       </c>
       <c r="E57" s="8" t="inlineStr">
         <is>
-          <t>-</t>
+          <t>Phase 8 follow-up</t>
         </is>
       </c>
       <c r="F57" s="8" t="inlineStr">
         <is>
-          <t>Superseded: see P7 for the current, generalized version of this story (LMX leadership routing to the cheapest eligible capacity, including gig couriers).</t>
+          <t>As the person receiving a delivery, I want a link that shows my driver's live position and ETA, so that I don't have to call the shop or guess when my part will arrive.</t>
         </is>
       </c>
     </row>
     <row r="58">
       <c r="A58" s="5" t="inlineStr">
         <is>
-          <t>F10</t>
+          <t>F4</t>
         </is>
       </c>
       <c r="B58" s="6" t="inlineStr">
@@ -2468,7 +2468,7 @@
       </c>
       <c r="C58" s="6" t="inlineStr">
         <is>
-          <t>A real path to SOC 2 (or equivalent) certification</t>
+          <t>Outbound status webhooks + integrations surface</t>
         </is>
       </c>
       <c r="D58" s="5" t="inlineStr">
@@ -2478,19 +2478,19 @@
       </c>
       <c r="E58" s="6" t="inlineStr">
         <is>
-          <t>Phase 5</t>
+          <t>Phase 8 follow-up</t>
         </is>
       </c>
       <c r="F58" s="6" t="inlineStr">
         <is>
-          <t>As an enterprise client's security team, I want to see a SOC 2 report before signing, so that I have independent assurance LMX handles data and access responsibly.</t>
+          <t>As a client's system administrator, I want to subscribe to order status webhooks, so that my own systems update automatically instead of polling or waiting on a manual check.</t>
         </is>
       </c>
     </row>
     <row r="59">
       <c r="A59" s="7" t="inlineStr">
         <is>
-          <t>F11</t>
+          <t>F5</t>
         </is>
       </c>
       <c r="B59" s="8" t="inlineStr">
@@ -2500,7 +2500,7 @@
       </c>
       <c r="C59" s="8" t="inlineStr">
         <is>
-          <t>SSO/SAML for ops and client logins</t>
+          <t>Flexible/rate-table billing</t>
         </is>
       </c>
       <c r="D59" s="7" t="inlineStr">
@@ -2510,19 +2510,19 @@
       </c>
       <c r="E59" s="8" t="inlineStr">
         <is>
-          <t>Phase 5</t>
+          <t>Phase 8 follow-up</t>
         </is>
       </c>
       <c r="F59" s="8" t="inlineStr">
         <is>
-          <t>As an enterprise client's IT admin, I want to enforce SSO for anyone accessing the portal, so that portal access follows the same identity policy as the rest of my company's tools.</t>
+          <t>As a client with orders of very different sizes, I want billing that can reflect piece count, weight, or mileage, not just a flat per-drop rate, so that pricing matches the actual cost of serving my orders.</t>
         </is>
       </c>
     </row>
     <row r="60">
       <c r="A60" s="5" t="inlineStr">
         <is>
-          <t>F12</t>
+          <t>F6</t>
         </is>
       </c>
       <c r="B60" s="6" t="inlineStr">
@@ -2532,7 +2532,7 @@
       </c>
       <c r="C60" s="6" t="inlineStr">
         <is>
-          <t>Network/territory optimization tooling</t>
+          <t>Real-time mid-route re-optimization</t>
         </is>
       </c>
       <c r="D60" s="5" t="inlineStr">
@@ -2542,19 +2542,19 @@
       </c>
       <c r="E60" s="6" t="inlineStr">
         <is>
-          <t>Later, multi-hub</t>
+          <t>Phase 4 (needs E1)</t>
         </is>
       </c>
       <c r="F60" s="6" t="inlineStr">
         <is>
-          <t>As LMX leadership planning a second or third hub, I want tooling to redesign depot/zone boundaries, so that expansion decisions are based on a real optimization model instead of intuition.</t>
+          <t>As a hub dispatcher, I want the optimizer to re-sequence an in-progress route when conditions change, so that a driver isn't stuck following a plan that's gone stale since the last cycle.</t>
         </is>
       </c>
     </row>
     <row r="61">
       <c r="A61" s="7" t="inlineStr">
         <is>
-          <t>F13</t>
+          <t>F7</t>
         </is>
       </c>
       <c r="B61" s="8" t="inlineStr">
@@ -2564,7 +2564,7 @@
       </c>
       <c r="C61" s="8" t="inlineStr">
         <is>
-          <t>Ratings &amp; feedback capture</t>
+          <t>Client- and ops-facing analytics dashboards</t>
         </is>
       </c>
       <c r="D61" s="7" t="inlineStr">
@@ -2574,19 +2574,19 @@
       </c>
       <c r="E61" s="8" t="inlineStr">
         <is>
-          <t>Phase 8 follow-up</t>
+          <t>Phase 10 (folds into I4)</t>
         </is>
       </c>
       <c r="F61" s="8" t="inlineStr">
         <is>
-          <t>As a shop after a delivery, I want to leave a quick rating and comment, so that LMX knows how the delivery actually went, not just whether the status says completed.</t>
+          <t>As a client company, I want to see my own on-time rate, volume, and cost trend in the portal, so that I have concrete proof of the value of switching to per-drop pricing with LMX.</t>
         </is>
       </c>
     </row>
     <row r="62">
       <c r="A62" s="5" t="inlineStr">
         <is>
-          <t>F14</t>
+          <t>F8</t>
         </is>
       </c>
       <c r="B62" s="6" t="inlineStr">
@@ -2596,7 +2596,7 @@
       </c>
       <c r="C62" s="6" t="inlineStr">
         <is>
-          <t>Orchestrator route-preview / shadow mode</t>
+          <t>White-label / multi-brand portal theming</t>
         </is>
       </c>
       <c r="D62" s="5" t="inlineStr">
@@ -2606,61 +2606,61 @@
       </c>
       <c r="E62" s="6" t="inlineStr">
         <is>
-          <t>Phase 9</t>
+          <t>Phase 8 follow-up</t>
         </is>
       </c>
       <c r="F62" s="6" t="inlineStr">
         <is>
-          <t>As a hub dispatcher during the pilot, I want to preview the optimizer's proposed plan and override it if needed, so that I can build trust in autonomous dispatch before relying on it fully.</t>
+          <t>As a reselling partner, I want the client portal to carry my own brand, so that my customers experience it as part of my business, not a visibly third-party tool.</t>
         </is>
       </c>
     </row>
     <row r="63">
       <c r="A63" s="7" t="inlineStr">
         <is>
-          <t>I1</t>
+          <t>F9</t>
         </is>
       </c>
       <c r="B63" s="8" t="inlineStr">
         <is>
-          <t>Intelligence layer</t>
+          <t>Competitive gaps</t>
         </is>
       </c>
       <c r="C63" s="8" t="inlineStr">
         <is>
-          <t>Ground-truth event capture</t>
-        </is>
-      </c>
-      <c r="D63" s="7" t="inlineStr">
-        <is>
-          <t>Open</t>
+          <t>Hybrid gig-fleet overflow dispatch</t>
+        </is>
+      </c>
+      <c r="D63" s="13" t="inlineStr">
+        <is>
+          <t>Superseded -&gt; reinstated as P7</t>
         </is>
       </c>
       <c r="E63" s="8" t="inlineStr">
         <is>
-          <t>Phase 10 (pre-pilot)</t>
+          <t>-</t>
         </is>
       </c>
       <c r="F63" s="8" t="inlineStr">
         <is>
-          <t>As the Learning Loop, I want real delivered/arrived timestamps and decline/hold-release data captured, so that there's actual ground truth to learn from instead of a proxy that was never meant for this.</t>
+          <t>Superseded: see P7 for the current, generalized version of this story (LMX leadership routing to the cheapest eligible capacity, including gig couriers).</t>
         </is>
       </c>
     </row>
     <row r="64">
       <c r="A64" s="5" t="inlineStr">
         <is>
-          <t>I2</t>
+          <t>F10</t>
         </is>
       </c>
       <c r="B64" s="6" t="inlineStr">
         <is>
-          <t>Intelligence layer</t>
+          <t>Competitive gaps</t>
         </is>
       </c>
       <c r="C64" s="6" t="inlineStr">
         <is>
-          <t>Rule review &amp; promotion flow</t>
+          <t>A real path to SOC 2 (or equivalent) certification</t>
         </is>
       </c>
       <c r="D64" s="5" t="inlineStr">
@@ -2670,29 +2670,29 @@
       </c>
       <c r="E64" s="6" t="inlineStr">
         <is>
-          <t>Phase 10 (pre-pilot)</t>
+          <t>Phase 5</t>
         </is>
       </c>
       <c r="F64" s="6" t="inlineStr">
         <is>
-          <t>As a hub ops manager, I want to review and approve or dismiss a proposed rule change from the Learning Loop, so that per-shop overrides get vetted by a person before they take effect.</t>
+          <t>As an enterprise client's security team, I want to see a SOC 2 report before signing, so that I have independent assurance LMX handles data and access responsibly.</t>
         </is>
       </c>
     </row>
     <row r="65">
       <c r="A65" s="7" t="inlineStr">
         <is>
-          <t>I3</t>
+          <t>F11</t>
         </is>
       </c>
       <c r="B65" s="8" t="inlineStr">
         <is>
-          <t>Intelligence layer</t>
+          <t>Competitive gaps</t>
         </is>
       </c>
       <c r="C65" s="8" t="inlineStr">
         <is>
-          <t>Broaden the annotation vocabulary</t>
+          <t>SSO/SAML for ops and client logins</t>
         </is>
       </c>
       <c r="D65" s="7" t="inlineStr">
@@ -2702,29 +2702,29 @@
       </c>
       <c r="E65" s="8" t="inlineStr">
         <is>
-          <t>Phase 10 (pre-pilot)</t>
+          <t>Phase 5</t>
         </is>
       </c>
       <c r="F65" s="8" t="inlineStr">
         <is>
-          <t>As a driver, I want to flag more than just hold-window issues (parking, gate codes, shop prep slowness), so that what I know about a shop becomes part of the system instead of staying in my head.</t>
+          <t>As an enterprise client's IT admin, I want to enforce SSO for anyone accessing the portal, so that portal access follows the same identity policy as the rest of my company's tools.</t>
         </is>
       </c>
     </row>
     <row r="66">
       <c r="A66" s="5" t="inlineStr">
         <is>
-          <t>I4</t>
+          <t>F12</t>
         </is>
       </c>
       <c r="B66" s="6" t="inlineStr">
         <is>
-          <t>Intelligence layer</t>
+          <t>Competitive gaps</t>
         </is>
       </c>
       <c r="C66" s="6" t="inlineStr">
         <is>
-          <t>Descriptive analytics on the captured truth</t>
+          <t>Network/territory optimization tooling</t>
         </is>
       </c>
       <c r="D66" s="5" t="inlineStr">
@@ -2734,83 +2734,83 @@
       </c>
       <c r="E66" s="6" t="inlineStr">
         <is>
-          <t>Phase 10 (during/after pilot)</t>
+          <t>Later, multi-hub</t>
         </is>
       </c>
       <c r="F66" s="6" t="inlineStr">
         <is>
-          <t>As a hub ops manager, I want DPH, SLA hit rate, and hold-window effectiveness reported per driver/hub/day, so that I can see how the operation is actually performing, not just whether the day went fine.</t>
+          <t>As LMX leadership planning a second or third hub, I want tooling to redesign depot/zone boundaries, so that expansion decisions are based on a real optimization model instead of intuition.</t>
         </is>
       </c>
     </row>
     <row r="67">
       <c r="A67" s="7" t="inlineStr">
         <is>
-          <t>I5</t>
+          <t>F13</t>
         </is>
       </c>
       <c r="B67" s="8" t="inlineStr">
         <is>
-          <t>Intelligence layer</t>
+          <t>Competitive gaps</t>
         </is>
       </c>
       <c r="C67" s="8" t="inlineStr">
         <is>
-          <t>Calibration from data</t>
+          <t>Ratings &amp; feedback capture</t>
         </is>
       </c>
       <c r="D67" s="7" t="inlineStr">
         <is>
-          <t>Open (=E2/E5/E9/E10)</t>
+          <t>Open</t>
         </is>
       </c>
       <c r="E67" s="8" t="inlineStr">
         <is>
-          <t>Phase 10 (during/after pilot)</t>
+          <t>Phase 8 follow-up</t>
         </is>
       </c>
       <c r="F67" s="8" t="inlineStr">
         <is>
-          <t>As LMX leadership, I want skip penalties, hold windows, and the DPH figure retuned from real data, so that every placeholder number gets replaced with something proven.</t>
+          <t>As a shop after a delivery, I want to leave a quick rating and comment, so that LMX knows how the delivery actually went, not just whether the status says completed.</t>
         </is>
       </c>
     </row>
     <row r="68">
       <c r="A68" s="5" t="inlineStr">
         <is>
-          <t>I6</t>
+          <t>F14</t>
         </is>
       </c>
       <c r="B68" s="6" t="inlineStr">
         <is>
-          <t>Intelligence layer</t>
+          <t>Competitive gaps</t>
         </is>
       </c>
       <c r="C68" s="6" t="inlineStr">
         <is>
-          <t>Predictive models</t>
+          <t>Orchestrator route-preview / shadow mode</t>
         </is>
       </c>
       <c r="D68" s="5" t="inlineStr">
         <is>
-          <t>Open (data-gated)</t>
+          <t>Open</t>
         </is>
       </c>
       <c r="E68" s="6" t="inlineStr">
         <is>
-          <t>Phase 10 (later)</t>
+          <t>Phase 9</t>
         </is>
       </c>
       <c r="F68" s="6" t="inlineStr">
         <is>
-          <t>As a hub dispatcher, I want the optimizer to use predicted ETAs and per-shop service times instead of static estimates, so that routes reflect what's actually likely to happen, not a fixed assumption.</t>
+          <t>As a hub dispatcher during the pilot, I want to preview the optimizer's proposed plan and override it if needed, so that I can build trust in autonomous dispatch before relying on it fully.</t>
         </is>
       </c>
     </row>
     <row r="69">
       <c r="A69" s="7" t="inlineStr">
         <is>
-          <t>I7</t>
+          <t>I1</t>
         </is>
       </c>
       <c r="B69" s="8" t="inlineStr">
@@ -2820,91 +2820,283 @@
       </c>
       <c r="C69" s="8" t="inlineStr">
         <is>
-          <t>Ops copilot</t>
+          <t>Ground-truth event capture</t>
         </is>
       </c>
       <c r="D69" s="7" t="inlineStr">
         <is>
-          <t>Open (needs LLM API key)</t>
+          <t>Open</t>
         </is>
       </c>
       <c r="E69" s="8" t="inlineStr">
         <is>
-          <t>Phase 10 (later)</t>
+          <t>Phase 10 (pre-pilot)</t>
         </is>
       </c>
       <c r="F69" s="8" t="inlineStr">
         <is>
-          <t>As a hub ops manager, I want to ask a natural-language question like 'why was yesterday slow?' and get a real answer from the system's own data, so that I don't have to manually dig through dashboards to explain a bad day.</t>
+          <t>As the Learning Loop, I want real delivered/arrived timestamps and decline/hold-release data captured, so that there's actual ground truth to learn from instead of a proxy that was never meant for this.</t>
         </is>
       </c>
     </row>
     <row r="70">
       <c r="A70" s="5" t="inlineStr">
         <is>
-          <t>T1</t>
+          <t>I2</t>
         </is>
       </c>
       <c r="B70" s="6" t="inlineStr">
         <is>
-          <t>Testing/process</t>
+          <t>Intelligence layer</t>
         </is>
       </c>
       <c r="C70" s="6" t="inlineStr">
         <is>
-          <t>Load/performance test against the design budget</t>
-        </is>
-      </c>
-      <c r="D70" s="10" t="inlineStr">
-        <is>
-          <t>Done</t>
+          <t>Rule review &amp; promotion flow</t>
+        </is>
+      </c>
+      <c r="D70" s="5" t="inlineStr">
+        <is>
+          <t>Open</t>
         </is>
       </c>
       <c r="E70" s="6" t="inlineStr">
         <is>
-          <t>Phase 9</t>
+          <t>Phase 10 (pre-pilot)</t>
         </is>
       </c>
       <c r="F70" s="6" t="inlineStr">
         <is>
-          <t>As the engineering team, I want the optimizer load-tested against the design budget (20 drivers/100 orders/&lt;5s), so that we know the dispatch cycle holds up before it's carrying real orders.</t>
+          <t>As a hub ops manager, I want to review and approve or dismiss a proposed rule change from the Learning Loop, so that per-shop overrides get vetted by a person before they take effect.</t>
         </is>
       </c>
     </row>
     <row r="71">
       <c r="A71" s="7" t="inlineStr">
         <is>
+          <t>I3</t>
+        </is>
+      </c>
+      <c r="B71" s="8" t="inlineStr">
+        <is>
+          <t>Intelligence layer</t>
+        </is>
+      </c>
+      <c r="C71" s="8" t="inlineStr">
+        <is>
+          <t>Broaden the annotation vocabulary</t>
+        </is>
+      </c>
+      <c r="D71" s="7" t="inlineStr">
+        <is>
+          <t>Open</t>
+        </is>
+      </c>
+      <c r="E71" s="8" t="inlineStr">
+        <is>
+          <t>Phase 10 (pre-pilot)</t>
+        </is>
+      </c>
+      <c r="F71" s="8" t="inlineStr">
+        <is>
+          <t>As a driver, I want to flag more than just hold-window issues (parking, gate codes, shop prep slowness), so that what I know about a shop becomes part of the system instead of staying in my head.</t>
+        </is>
+      </c>
+    </row>
+    <row r="72">
+      <c r="A72" s="5" t="inlineStr">
+        <is>
+          <t>I4</t>
+        </is>
+      </c>
+      <c r="B72" s="6" t="inlineStr">
+        <is>
+          <t>Intelligence layer</t>
+        </is>
+      </c>
+      <c r="C72" s="6" t="inlineStr">
+        <is>
+          <t>Descriptive analytics on the captured truth</t>
+        </is>
+      </c>
+      <c r="D72" s="5" t="inlineStr">
+        <is>
+          <t>Open</t>
+        </is>
+      </c>
+      <c r="E72" s="6" t="inlineStr">
+        <is>
+          <t>Phase 10 (during/after pilot)</t>
+        </is>
+      </c>
+      <c r="F72" s="6" t="inlineStr">
+        <is>
+          <t>As a hub ops manager, I want DPH, SLA hit rate, and hold-window effectiveness reported per driver/hub/day, so that I can see how the operation is actually performing, not just whether the day went fine.</t>
+        </is>
+      </c>
+    </row>
+    <row r="73">
+      <c r="A73" s="7" t="inlineStr">
+        <is>
+          <t>I5</t>
+        </is>
+      </c>
+      <c r="B73" s="8" t="inlineStr">
+        <is>
+          <t>Intelligence layer</t>
+        </is>
+      </c>
+      <c r="C73" s="8" t="inlineStr">
+        <is>
+          <t>Calibration from data</t>
+        </is>
+      </c>
+      <c r="D73" s="7" t="inlineStr">
+        <is>
+          <t>Open (=E2/E5/E9/E10)</t>
+        </is>
+      </c>
+      <c r="E73" s="8" t="inlineStr">
+        <is>
+          <t>Phase 10 (during/after pilot)</t>
+        </is>
+      </c>
+      <c r="F73" s="8" t="inlineStr">
+        <is>
+          <t>As LMX leadership, I want skip penalties, hold windows, and the DPH figure retuned from real data, so that every placeholder number gets replaced with something proven.</t>
+        </is>
+      </c>
+    </row>
+    <row r="74">
+      <c r="A74" s="5" t="inlineStr">
+        <is>
+          <t>I6</t>
+        </is>
+      </c>
+      <c r="B74" s="6" t="inlineStr">
+        <is>
+          <t>Intelligence layer</t>
+        </is>
+      </c>
+      <c r="C74" s="6" t="inlineStr">
+        <is>
+          <t>Predictive models</t>
+        </is>
+      </c>
+      <c r="D74" s="5" t="inlineStr">
+        <is>
+          <t>Open (data-gated)</t>
+        </is>
+      </c>
+      <c r="E74" s="6" t="inlineStr">
+        <is>
+          <t>Phase 10 (later)</t>
+        </is>
+      </c>
+      <c r="F74" s="6" t="inlineStr">
+        <is>
+          <t>As a hub dispatcher, I want the optimizer to use predicted ETAs and per-shop service times instead of static estimates, so that routes reflect what's actually likely to happen, not a fixed assumption.</t>
+        </is>
+      </c>
+    </row>
+    <row r="75">
+      <c r="A75" s="7" t="inlineStr">
+        <is>
+          <t>I7</t>
+        </is>
+      </c>
+      <c r="B75" s="8" t="inlineStr">
+        <is>
+          <t>Intelligence layer</t>
+        </is>
+      </c>
+      <c r="C75" s="8" t="inlineStr">
+        <is>
+          <t>Ops copilot</t>
+        </is>
+      </c>
+      <c r="D75" s="7" t="inlineStr">
+        <is>
+          <t>Open (needs LLM API key)</t>
+        </is>
+      </c>
+      <c r="E75" s="8" t="inlineStr">
+        <is>
+          <t>Phase 10 (later)</t>
+        </is>
+      </c>
+      <c r="F75" s="8" t="inlineStr">
+        <is>
+          <t>As a hub ops manager, I want to ask a natural-language question like 'why was yesterday slow?' and get a real answer from the system's own data, so that I don't have to manually dig through dashboards to explain a bad day.</t>
+        </is>
+      </c>
+    </row>
+    <row r="76">
+      <c r="A76" s="5" t="inlineStr">
+        <is>
+          <t>T1</t>
+        </is>
+      </c>
+      <c r="B76" s="6" t="inlineStr">
+        <is>
+          <t>Testing/process</t>
+        </is>
+      </c>
+      <c r="C76" s="6" t="inlineStr">
+        <is>
+          <t>Load/performance test against the design budget</t>
+        </is>
+      </c>
+      <c r="D76" s="10" t="inlineStr">
+        <is>
+          <t>Done</t>
+        </is>
+      </c>
+      <c r="E76" s="6" t="inlineStr">
+        <is>
+          <t>Phase 9</t>
+        </is>
+      </c>
+      <c r="F76" s="6" t="inlineStr">
+        <is>
+          <t>As the engineering team, I want the optimizer load-tested against the design budget (20 drivers/100 orders/&lt;5s), so that we know the dispatch cycle holds up before it's carrying real orders.</t>
+        </is>
+      </c>
+    </row>
+    <row r="77">
+      <c r="A77" s="7" t="inlineStr">
+        <is>
           <t>T2</t>
         </is>
       </c>
-      <c r="B71" s="8" t="inlineStr">
+      <c r="B77" s="8" t="inlineStr">
         <is>
           <t>Testing/process</t>
         </is>
       </c>
-      <c r="C71" s="8" t="inlineStr">
+      <c r="C77" s="8" t="inlineStr">
         <is>
           <t>Local sandbox can't fully exercise Redis rate limiting</t>
         </is>
       </c>
-      <c r="D71" s="7" t="inlineStr">
+      <c r="D77" s="7" t="inlineStr">
         <is>
           <t>Documented, not a bug</t>
         </is>
       </c>
-      <c r="E71" s="8" t="inlineStr">
+      <c r="E77" s="8" t="inlineStr">
         <is>
           <t>-</t>
         </is>
       </c>
-      <c r="F71" s="8" t="inlineStr">
+      <c r="F77" s="8" t="inlineStr">
         <is>
           <t>As the engineering team, I want it documented that the sandbox's test Redis can't exercise EXPIRE...NX the way production Redis does, so that this known limitation doesn't get 'rediscovered' and mistaken for a real bug.</t>
         </is>
       </c>
     </row>
   </sheetData>
-  <autoFilter ref="A1:F71"/>
+  <autoFilter ref="A1:F77"/>
   <pageMargins left="0.75" right="0.75" top="1" bottom="1" header="0.5" footer="0.5"/>
 </worksheet>
 </file>
</xml_diff>

<commit_message>
Regenerate deliverables for the workflow-session reconciliation (76 -> 86 items)
Adds W1-W9 and I8 with persona-voiced user stories drawn from the
session doc itself where one existed. The readable roadmap doc picks up
the new Phase 3.5, the rewritten Phase 9, and a plain-language callout
explaining that Hub 1 launches on a scaffold rather than on LMX OS.

Cross-check clean: every roadmap item has a story row (C1/C2 remain
intentional spreadsheet-only rows for the shipped Phase 8 work).
</commit_message>
<xml_diff>
--- a/docs/LMX_OS_Roadmap_User_Stories.xlsx
+++ b/docs/LMX_OS_Roadmap_User_Stories.xlsx
@@ -11,7 +11,7 @@
     <sheet xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" name="User Stories" sheetId="2" state="visible" r:id="rId2"/>
   </sheets>
   <definedNames>
-    <definedName name="_xlnm._FilterDatabase" localSheetId="1" hidden="1">'User Stories'!$A$1:$F$77</definedName>
+    <definedName name="_xlnm._FilterDatabase" localSheetId="1" hidden="1">'User Stories'!$A$1:$F$87</definedName>
   </definedNames>
   <calcPr calcId="124519" fullCalcOnLoad="1"/>
 </workbook>
@@ -152,13 +152,13 @@
     <xf numFmtId="0" fontId="6" fillId="3" borderId="1" applyAlignment="1" pivotButton="0" quotePrefix="0" xfId="0">
       <alignment vertical="top" wrapText="1"/>
     </xf>
+    <xf numFmtId="0" fontId="7" fillId="0" borderId="1" applyAlignment="1" pivotButton="0" quotePrefix="0" xfId="0">
+      <alignment vertical="top" wrapText="1"/>
+    </xf>
     <xf numFmtId="0" fontId="7" fillId="3" borderId="1" applyAlignment="1" pivotButton="0" quotePrefix="0" xfId="0">
       <alignment vertical="top" wrapText="1"/>
     </xf>
-    <xf numFmtId="0" fontId="7" fillId="0" borderId="1" applyAlignment="1" pivotButton="0" quotePrefix="0" xfId="0">
-      <alignment vertical="top" wrapText="1"/>
-    </xf>
-    <xf numFmtId="0" fontId="8" fillId="0" borderId="1" applyAlignment="1" pivotButton="0" quotePrefix="0" xfId="0">
+    <xf numFmtId="0" fontId="8" fillId="3" borderId="1" applyAlignment="1" pivotButton="0" quotePrefix="0" xfId="0">
       <alignment vertical="top" wrapText="1"/>
     </xf>
   </cellXfs>
@@ -620,7 +620,7 @@
     <outlinePr summaryBelow="1" summaryRight="1"/>
     <pageSetUpPr/>
   </sheetPr>
-  <dimension ref="A1:F77"/>
+  <dimension ref="A1:F87"/>
   <sheetFormatPr baseColWidth="8" defaultRowHeight="15"/>
   <cols>
     <col width="7" customWidth="1" min="1" max="1"/>
@@ -826,113 +826,113 @@
     <row r="7">
       <c r="A7" s="7" t="inlineStr">
         <is>
-          <t>R1</t>
+          <t>W1</t>
         </is>
       </c>
       <c r="B7" s="8" t="inlineStr">
         <is>
-          <t>Risk &amp; compliance</t>
+          <t>Workflow gaps</t>
         </is>
       </c>
       <c r="C7" s="8" t="inlineStr">
         <is>
-          <t>Insurance &amp; liability plan</t>
+          <t>Returns &amp; core pickups as first-class work</t>
         </is>
       </c>
       <c r="D7" s="7" t="inlineStr">
         <is>
-          <t>Open - gates Phase 9</t>
+          <t>Open</t>
         </is>
       </c>
       <c r="E7" s="8" t="inlineStr">
         <is>
-          <t>Start now (business/legal)</t>
+          <t>Phase 6</t>
         </is>
       </c>
       <c r="F7" s="8" t="inlineStr">
         <is>
-          <t>As LMX leadership, I want commercial auto, cargo, and general liability coverage in place before drivers carry real packages, so that a single accident or lost shipment is an insured event rather than a company-ending liability.</t>
+          <t>As a shop owner, I want the driver to collect my tagged cores and returns during the delivery stop and confirm what was taken, so that my credits move as fast as my parts - and as a driver, I want those pickups to appear as real route stops with an item list, so that every kind of work I do is counted work.</t>
         </is>
       </c>
     </row>
     <row r="8">
       <c r="A8" s="5" t="inlineStr">
         <is>
-          <t>R2</t>
+          <t>W2</t>
         </is>
       </c>
       <c r="B8" s="6" t="inlineStr">
         <is>
-          <t>Risk &amp; compliance</t>
+          <t>Workflow gaps</t>
         </is>
       </c>
       <c r="C8" s="6" t="inlineStr">
         <is>
-          <t>Driver background checks &amp; MVR screening</t>
+          <t>COD collection &amp; payment disputes</t>
         </is>
       </c>
       <c r="D8" s="5" t="inlineStr">
         <is>
-          <t>Open - gates Phase 9</t>
+          <t>Open</t>
         </is>
       </c>
       <c r="E8" s="6" t="inlineStr">
         <is>
-          <t>Start now (business/legal)</t>
+          <t>Phase 6</t>
         </is>
       </c>
       <c r="F8" s="6" t="inlineStr">
         <is>
-          <t>As LMX leadership, I want every driver background-checked and their motor-vehicle record screened before their first shift, so that we know a driver is safe to put on the road - document expiry tracking alone doesn't tell us that.</t>
+          <t>As a driver facing a customer who disputes the charge at the door, I want one tap to escalate to the distributor so I can keep moving, so that I never negotiate money on a doorstep - and as a distributor owner, I want accounts with repeated disputes surfaced monthly, so that I resolve money problems in my office, not at my customers' doors.</t>
         </is>
       </c>
     </row>
     <row r="9">
       <c r="A9" s="7" t="inlineStr">
         <is>
-          <t>R3</t>
+          <t>W3</t>
         </is>
       </c>
       <c r="B9" s="8" t="inlineStr">
         <is>
-          <t>Risk &amp; compliance</t>
+          <t>Workflow gaps</t>
         </is>
       </c>
       <c r="C9" s="8" t="inlineStr">
         <is>
-          <t>Privacy policy &amp; data-handling/retention policy</t>
+          <t>SLA-breach invoice credits</t>
         </is>
       </c>
       <c r="D9" s="7" t="inlineStr">
         <is>
-          <t>Open - gates Phase 9</t>
+          <t>Open</t>
         </is>
       </c>
       <c r="E9" s="8" t="inlineStr">
         <is>
-          <t>Start now (business/legal)</t>
+          <t>Phase 8 follow-up</t>
         </is>
       </c>
       <c r="F9" s="8" t="inlineStr">
         <is>
-          <t>As a customer whose name, address, and phone number LMX stores, I want a published policy saying what happens to my data and how I can have it deleted, so that my information is handled accountably - and so LMX can answer an enterprise client's security questionnaire.</t>
+          <t>As a distributor owner, I want contractually defined invoice credits when SLA thresholds are breached, so that my delivery vendor is paid for outcomes rather than effort.</t>
         </is>
       </c>
     </row>
     <row r="10">
       <c r="A10" s="5" t="inlineStr">
         <is>
-          <t>R4</t>
+          <t>W4</t>
         </is>
       </c>
       <c r="B10" s="6" t="inlineStr">
         <is>
-          <t>Risk &amp; compliance</t>
+          <t>Workflow gaps</t>
         </is>
       </c>
       <c r="C10" s="6" t="inlineStr">
         <is>
-          <t>Driver document upload pipeline</t>
+          <t>Driver-visible scorecard</t>
         </is>
       </c>
       <c r="D10" s="5" t="inlineStr">
@@ -942,29 +942,29 @@
       </c>
       <c r="E10" s="6" t="inlineStr">
         <is>
-          <t>Phase 6 (with A3)</t>
+          <t>Phase 10 (with I4)</t>
         </is>
       </c>
       <c r="F10" s="6" t="inlineStr">
         <is>
-          <t>As LMX's onboarding staff, I want drivers to upload real license and insurance documents through the app, so that compliance evidence is a verified file on record rather than whatever text string was typed into the field.</t>
+          <t>As a driver, I want to see my own numbers in the same view and with the same definitions the company uses, so that the scorecard reads as a shared standard rather than a camera pointed at me.</t>
         </is>
       </c>
     </row>
     <row r="11">
       <c r="A11" s="7" t="inlineStr">
         <is>
-          <t>R5</t>
+          <t>W5</t>
         </is>
       </c>
       <c r="B11" s="8" t="inlineStr">
         <is>
-          <t>Risk &amp; compliance</t>
+          <t>Workflow gaps</t>
         </is>
       </c>
       <c r="C11" s="8" t="inlineStr">
         <is>
-          <t>Failed-delivery / redelivery workflow</t>
+          <t>Counter-person order status lookup</t>
         </is>
       </c>
       <c r="D11" s="7" t="inlineStr">
@@ -974,29 +974,29 @@
       </c>
       <c r="E11" s="8" t="inlineStr">
         <is>
-          <t>Phase 4</t>
+          <t>Phase 8 follow-up</t>
         </is>
       </c>
       <c r="F11" s="8" t="inlineStr">
         <is>
-          <t>As a hub dispatcher facing a refused package, wrong address, or closed shop, I want a defined path for what happens next - redelivery, client notification, billing adjustment - so that a failed order gets resolved instead of sitting in a dead-end status forever.</t>
+          <t>As a counter person, I want to look up any order's live status and ETA by shop name or order number, so that the rare status question takes ten seconds instead of a radio call.</t>
         </is>
       </c>
     </row>
     <row r="12">
       <c r="A12" s="5" t="inlineStr">
         <is>
-          <t>R6</t>
+          <t>W6</t>
         </is>
       </c>
       <c r="B12" s="6" t="inlineStr">
         <is>
-          <t>Risk &amp; compliance</t>
+          <t>Workflow gaps</t>
         </is>
       </c>
       <c r="C12" s="6" t="inlineStr">
         <is>
-          <t>Hub closure / holiday calendar</t>
+          <t>Orchestrator-editable urgency configuration</t>
         </is>
       </c>
       <c r="D12" s="5" t="inlineStr">
@@ -1006,61 +1006,61 @@
       </c>
       <c r="E12" s="6" t="inlineStr">
         <is>
-          <t>Phase 4</t>
+          <t>No dependency</t>
         </is>
       </c>
       <c r="F12" s="6" t="inlineStr">
         <is>
-          <t>As a hub ops manager, I want to mark days the hub isn't operating, so that the nightly learning job and the dispatch optimizer don't plan routes for a hub that's closed for a holiday or weather event.</t>
+          <t>As the orchestrator, I want to adjust part-type urgency rules myself in configuration, so that 'body panels are never urgent' doesn't require a developer and a deploy.</t>
         </is>
       </c>
     </row>
     <row r="13">
       <c r="A13" s="7" t="inlineStr">
         <is>
-          <t>E1</t>
+          <t>W7</t>
         </is>
       </c>
       <c r="B13" s="8" t="inlineStr">
         <is>
-          <t>Core backend</t>
+          <t>Workflow gaps</t>
         </is>
       </c>
       <c r="C13" s="8" t="inlineStr">
         <is>
-          <t>Verify Google Route Optimization against a live project</t>
+          <t>Training-data rights in the customer contract</t>
         </is>
       </c>
       <c r="D13" s="7" t="inlineStr">
         <is>
-          <t>Open</t>
+          <t>Open - gates B2</t>
         </is>
       </c>
       <c r="E13" s="8" t="inlineStr">
         <is>
-          <t>Phase 4</t>
+          <t>Now (legal)</t>
         </is>
       </c>
       <c r="F13" s="8" t="inlineStr">
         <is>
-          <t>As a hub dispatcher relying on the optimizer, I want the Google Route Optimization integration verified against a real API call, so that I can trust the routes it proposes instead of an unverified request/response mapping.</t>
+          <t>As LMX leadership, I want model-training rights, cross-customer aggregation rights, and anonymization terms written into customer #1's contract before the first delivery, so that the data the operation generates is usable for the learning loop without a later amendment.</t>
         </is>
       </c>
     </row>
     <row r="14">
       <c r="A14" s="5" t="inlineStr">
         <is>
-          <t>E2</t>
+          <t>W8</t>
         </is>
       </c>
       <c r="B14" s="6" t="inlineStr">
         <is>
-          <t>Core backend</t>
+          <t>Workflow gaps</t>
         </is>
       </c>
       <c r="C14" s="6" t="inlineStr">
         <is>
-          <t>Tune SLA_TIER_SKIP_PENALTY values</t>
+          <t>Epicor staging-module qualification check</t>
         </is>
       </c>
       <c r="D14" s="5" t="inlineStr">
@@ -1070,29 +1070,29 @@
       </c>
       <c r="E14" s="6" t="inlineStr">
         <is>
-          <t>Phase 4 / I5</t>
+          <t>Now (sales process)</t>
         </is>
       </c>
       <c r="F14" s="6" t="inlineStr">
         <is>
-          <t>As a hub dispatcher, I want the SLA tier skip penalties tuned to real route economics, so that the optimizer's tier prioritization reflects actual cost tradeoffs instead of a placeholder ordering.</t>
+          <t>As LMX's sales lead, I want to ask whether a prospect's Epicor runs a warehouse/staging module before signing, so that we know whether real-time ingestion is even possible for that customer rather than discovering it after the contract.</t>
         </is>
       </c>
     </row>
     <row r="15">
       <c r="A15" s="7" t="inlineStr">
         <is>
-          <t>E3</t>
+          <t>W9</t>
         </is>
       </c>
       <c r="B15" s="8" t="inlineStr">
         <is>
-          <t>Core backend</t>
+          <t>Workflow gaps</t>
         </is>
       </c>
       <c r="C15" s="8" t="inlineStr">
         <is>
-          <t>Confirm real Epicor payload field names</t>
+          <t>Shadow-mode comparison engine &amp; cutover scorecard</t>
         </is>
       </c>
       <c r="D15" s="7" t="inlineStr">
@@ -1102,189 +1102,189 @@
       </c>
       <c r="E15" s="8" t="inlineStr">
         <is>
-          <t>Phase 4 (needs B2)</t>
+          <t>Phase 9</t>
         </is>
       </c>
       <c r="F15" s="8" t="inlineStr">
         <is>
-          <t>As the engineer integrating with a client's Epicor system, I want the real payload field names confirmed against a live tenant, so that orders ingest correctly instead of failing on a guessed schema.</t>
+          <t>As a distributor owner, I want LMX OS to run alongside my existing dispatch on my real orders for a few weeks before cutover, so that I see the performance gap on my own volume before I commit - measured on nine metrics with the divergent orders examined individually, not just the aggregates.</t>
         </is>
       </c>
     </row>
     <row r="16">
       <c r="A16" s="5" t="inlineStr">
         <is>
-          <t>E4</t>
+          <t>R1</t>
         </is>
       </c>
       <c r="B16" s="6" t="inlineStr">
         <is>
-          <t>Core backend</t>
+          <t>Risk &amp; compliance</t>
         </is>
       </c>
       <c r="C16" s="6" t="inlineStr">
         <is>
-          <t>Verify the batch-hold 4-question decision logic</t>
+          <t>Insurance &amp; liability plan</t>
         </is>
       </c>
       <c r="D16" s="5" t="inlineStr">
         <is>
-          <t>Open</t>
+          <t>Open - gates Phase 9</t>
         </is>
       </c>
       <c r="E16" s="6" t="inlineStr">
         <is>
-          <t>Phase 4 (needs B3)</t>
+          <t>Start now (business/legal)</t>
         </is>
       </c>
       <c r="F16" s="6" t="inlineStr">
         <is>
-          <t>As a hub dispatcher, I want the batch-hold decision logic verified against the canonical spec, so that commingling decisions match the intended design rather than a reconstructed interpretation.</t>
+          <t>As LMX leadership, I want commercial auto, cargo, and general liability coverage in place before drivers carry real packages, so that a single accident or lost shipment is an insured event rather than a company-ending liability.</t>
         </is>
       </c>
     </row>
     <row r="17">
       <c r="A17" s="7" t="inlineStr">
         <is>
-          <t>E5</t>
+          <t>R2</t>
         </is>
       </c>
       <c r="B17" s="8" t="inlineStr">
         <is>
-          <t>Core backend</t>
+          <t>Risk &amp; compliance</t>
         </is>
       </c>
       <c r="C17" s="8" t="inlineStr">
         <is>
-          <t>Recalibrate SLA hold-window minutes</t>
+          <t>Driver background checks &amp; MVR screening</t>
         </is>
       </c>
       <c r="D17" s="7" t="inlineStr">
         <is>
-          <t>Open</t>
+          <t>Open - gates Phase 9</t>
         </is>
       </c>
       <c r="E17" s="8" t="inlineStr">
         <is>
-          <t>Phase 4 / I5</t>
+          <t>Start now (business/legal)</t>
         </is>
       </c>
       <c r="F17" s="8" t="inlineStr">
         <is>
-          <t>As a hub dispatcher, I want the SLA hold-window minutes recalibrated from real Hub 1 data, so that orders are held just long enough to batch efficiently without risking an SLA breach.</t>
+          <t>As LMX leadership, I want every driver background-checked and their motor-vehicle record screened before their first shift, so that we know a driver is safe to put on the road - document expiry tracking alone doesn't tell us that.</t>
         </is>
       </c>
     </row>
     <row r="18">
       <c r="A18" s="5" t="inlineStr">
         <is>
-          <t>E6</t>
+          <t>R3</t>
         </is>
       </c>
       <c r="B18" s="6" t="inlineStr">
         <is>
-          <t>Core backend</t>
+          <t>Risk &amp; compliance</t>
         </is>
       </c>
       <c r="C18" s="6" t="inlineStr">
         <is>
-          <t>Confirm Learning Loop flag-type naming convention</t>
+          <t>Privacy policy &amp; data-handling/retention policy</t>
         </is>
       </c>
       <c r="D18" s="5" t="inlineStr">
         <is>
-          <t>Open</t>
+          <t>Open - gates Phase 9</t>
         </is>
       </c>
       <c r="E18" s="6" t="inlineStr">
         <is>
-          <t>Phase 4</t>
+          <t>Start now (business/legal)</t>
         </is>
       </c>
       <c r="F18" s="6" t="inlineStr">
         <is>
-          <t>As the engineer building the annotation loop, I want the flag-type naming convention signed off by a driver-app stakeholder, so that the contract between driver annotations and the Learning Loop isn't just an internal guess.</t>
+          <t>As a customer whose name, address, and phone number LMX stores, I want a published policy saying what happens to my data and how I can have it deleted, so that my information is handled accountably - and so LMX can answer an enterprise client's security questionnaire.</t>
         </is>
       </c>
     </row>
     <row r="19">
       <c r="A19" s="7" t="inlineStr">
         <is>
-          <t>E7</t>
+          <t>R4</t>
         </is>
       </c>
       <c r="B19" s="8" t="inlineStr">
         <is>
-          <t>Core backend</t>
+          <t>Risk &amp; compliance</t>
         </is>
       </c>
       <c r="C19" s="8" t="inlineStr">
         <is>
-          <t>Wire a real scheduler for the Learning Loop's nightly job</t>
-        </is>
-      </c>
-      <c r="D19" s="9" t="inlineStr">
-        <is>
-          <t>Done</t>
+          <t>Driver document upload pipeline</t>
+        </is>
+      </c>
+      <c r="D19" s="7" t="inlineStr">
+        <is>
+          <t>Open</t>
         </is>
       </c>
       <c r="E19" s="8" t="inlineStr">
         <is>
-          <t>Phase 4</t>
+          <t>Phase 6 (with A3)</t>
         </is>
       </c>
       <c r="F19" s="8" t="inlineStr">
         <is>
-          <t>As a hub, I want the Learning Loop's nightly detection job to run automatically on schedule, so that rule proposals get generated every night without anyone manually triggering it.</t>
+          <t>As LMX's onboarding staff, I want drivers to upload real license and insurance documents through the app, so that compliance evidence is a verified file on record rather than whatever text string was typed into the field.</t>
         </is>
       </c>
     </row>
     <row r="20">
       <c r="A20" s="5" t="inlineStr">
         <is>
-          <t>E8</t>
+          <t>R5</t>
         </is>
       </c>
       <c r="B20" s="6" t="inlineStr">
         <is>
-          <t>Core backend</t>
+          <t>Risk &amp; compliance</t>
         </is>
       </c>
       <c r="C20" s="6" t="inlineStr">
         <is>
-          <t>Move the event bus off in-process</t>
-        </is>
-      </c>
-      <c r="D20" s="10" t="inlineStr">
-        <is>
-          <t>Done</t>
+          <t>Failed-delivery / redelivery workflow</t>
+        </is>
+      </c>
+      <c r="D20" s="5" t="inlineStr">
+        <is>
+          <t>Open</t>
         </is>
       </c>
       <c r="E20" s="6" t="inlineStr">
         <is>
-          <t>Phase 5</t>
+          <t>Phase 4</t>
         </is>
       </c>
       <c r="F20" s="6" t="inlineStr">
         <is>
-          <t>As the platform running on more than one instance, I want the event bus backed by Redis instead of in-process memory, so that hold-release and dispatch events stay consistent across multiple app instances.</t>
+          <t>As a hub dispatcher facing a refused package, wrong address, or closed shop, I want a defined path for what happens next - redelivery, client notification, billing adjustment - so that a failed order gets resolved instead of sitting in a dead-end status forever.</t>
         </is>
       </c>
     </row>
     <row r="21">
       <c r="A21" s="7" t="inlineStr">
         <is>
-          <t>E9</t>
+          <t>R6</t>
         </is>
       </c>
       <c r="B21" s="8" t="inlineStr">
         <is>
-          <t>Core backend</t>
+          <t>Risk &amp; compliance</t>
         </is>
       </c>
       <c r="C21" s="8" t="inlineStr">
         <is>
-          <t>Validate the 2.5 DPH figure</t>
+          <t>Hub closure / holiday calendar</t>
         </is>
       </c>
       <c r="D21" s="7" t="inlineStr">
@@ -1294,19 +1294,19 @@
       </c>
       <c r="E21" s="8" t="inlineStr">
         <is>
-          <t>Phase 9 (needs B2)</t>
+          <t>Phase 4</t>
         </is>
       </c>
       <c r="F21" s="8" t="inlineStr">
         <is>
-          <t>As LMX leadership, I want the 2.5 deliveries-per-hour assumption validated against real Hub 1 data, so that pricing and staffing decisions rest on a proven number instead of a model assumption.</t>
+          <t>As a hub ops manager, I want to mark days the hub isn't operating, so that the nightly learning job and the dispatch optimizer don't plan routes for a hub that's closed for a holiday or weather event.</t>
         </is>
       </c>
     </row>
     <row r="22">
       <c r="A22" s="5" t="inlineStr">
         <is>
-          <t>E10</t>
+          <t>E1</t>
         </is>
       </c>
       <c r="B22" s="6" t="inlineStr">
@@ -1316,7 +1316,7 @@
       </c>
       <c r="C22" s="6" t="inlineStr">
         <is>
-          <t>Tune HOT_SHOT's skip-penalty/hold-window placeholders</t>
+          <t>Verify Google Route Optimization against a live project</t>
         </is>
       </c>
       <c r="D22" s="5" t="inlineStr">
@@ -1326,61 +1326,61 @@
       </c>
       <c r="E22" s="6" t="inlineStr">
         <is>
-          <t>Phase 8 follow-up / I5</t>
+          <t>Phase 4</t>
         </is>
       </c>
       <c r="F22" s="6" t="inlineStr">
         <is>
-          <t>As a hub dispatcher, I want HOT_SHOT's skip-penalty and hold-window values calibrated like the other tiers, so that the premium tier's priority handling is based on real economics, not a guess.</t>
+          <t>As a hub dispatcher relying on the optimizer, I want the Google Route Optimization integration verified against a real API call, so that I can trust the routes it proposes instead of an unverified request/response mapping.</t>
         </is>
       </c>
     </row>
     <row r="23">
       <c r="A23" s="7" t="inlineStr">
         <is>
-          <t>S1</t>
+          <t>E2</t>
         </is>
       </c>
       <c r="B23" s="8" t="inlineStr">
         <is>
-          <t>Security</t>
+          <t>Core backend</t>
         </is>
       </c>
       <c r="C23" s="8" t="inlineStr">
         <is>
-          <t>Real per-user authentication for the ops dashboard</t>
-        </is>
-      </c>
-      <c r="D23" s="9" t="inlineStr">
-        <is>
-          <t>Done</t>
+          <t>Tune SLA_TIER_SKIP_PENALTY values</t>
+        </is>
+      </c>
+      <c r="D23" s="7" t="inlineStr">
+        <is>
+          <t>Open</t>
         </is>
       </c>
       <c r="E23" s="8" t="inlineStr">
         <is>
-          <t>Phase 5</t>
+          <t>Phase 4 / I5</t>
         </is>
       </c>
       <c r="F23" s="8" t="inlineStr">
         <is>
-          <t>As a hub ops manager, I want each staff member to log in with their own account and role, so that I know who did what in the dashboard and can limit admin actions to admins.</t>
+          <t>As a hub dispatcher, I want the SLA tier skip penalties tuned to real route economics, so that the optimizer's tier prioritization reflects actual cost tradeoffs instead of a placeholder ordering.</t>
         </is>
       </c>
     </row>
     <row r="24">
       <c r="A24" s="5" t="inlineStr">
         <is>
-          <t>S2</t>
+          <t>E3</t>
         </is>
       </c>
       <c r="B24" s="6" t="inlineStr">
         <is>
-          <t>Security</t>
+          <t>Core backend</t>
         </is>
       </c>
       <c r="C24" s="6" t="inlineStr">
         <is>
-          <t>Secrets management</t>
+          <t>Confirm real Epicor payload field names</t>
         </is>
       </c>
       <c r="D24" s="5" t="inlineStr">
@@ -1390,29 +1390,29 @@
       </c>
       <c r="E24" s="6" t="inlineStr">
         <is>
-          <t>Phase 5</t>
+          <t>Phase 4 (needs B2)</t>
         </is>
       </c>
       <c r="F24" s="6" t="inlineStr">
         <is>
-          <t>As the engineering team, I want credentials stored in a real secrets manager instead of a .env file, so that a leaked file or repo doesn't hand over database passwords and API keys.</t>
+          <t>As the engineer integrating with a client's Epicor system, I want the real payload field names confirmed against a live tenant, so that orders ingest correctly instead of failing on a guessed schema.</t>
         </is>
       </c>
     </row>
     <row r="25">
       <c r="A25" s="7" t="inlineStr">
         <is>
-          <t>S3</t>
+          <t>E4</t>
         </is>
       </c>
       <c r="B25" s="8" t="inlineStr">
         <is>
-          <t>Security</t>
+          <t>Core backend</t>
         </is>
       </c>
       <c r="C25" s="8" t="inlineStr">
         <is>
-          <t>A real production hosting decision</t>
+          <t>Verify the batch-hold 4-question decision logic</t>
         </is>
       </c>
       <c r="D25" s="7" t="inlineStr">
@@ -1422,125 +1422,125 @@
       </c>
       <c r="E25" s="8" t="inlineStr">
         <is>
-          <t>Phase 5</t>
+          <t>Phase 4 (needs B3)</t>
         </is>
       </c>
       <c r="F25" s="8" t="inlineStr">
         <is>
-          <t>As the engineering team preparing for Hub 1, I want a resilient hosting setup instead of a single-instance docker-compose, so that a container crash or server failure doesn't take down dispatch for real drivers and orders.</t>
+          <t>As a hub dispatcher, I want the batch-hold decision logic verified against the canonical spec, so that commingling decisions match the intended design rather than a reconstructed interpretation.</t>
         </is>
       </c>
     </row>
     <row r="26">
       <c r="A26" s="5" t="inlineStr">
         <is>
-          <t>S4</t>
+          <t>E5</t>
         </is>
       </c>
       <c r="B26" s="6" t="inlineStr">
         <is>
-          <t>Security</t>
+          <t>Core backend</t>
         </is>
       </c>
       <c r="C26" s="6" t="inlineStr">
         <is>
-          <t>Observability</t>
-        </is>
-      </c>
-      <c r="D26" s="11" t="inlineStr">
-        <is>
-          <t>Partial</t>
+          <t>Recalibrate SLA hold-window minutes</t>
+        </is>
+      </c>
+      <c r="D26" s="5" t="inlineStr">
+        <is>
+          <t>Open</t>
         </is>
       </c>
       <c r="E26" s="6" t="inlineStr">
         <is>
-          <t>Phase 5</t>
+          <t>Phase 4 / I5</t>
         </is>
       </c>
       <c r="F26" s="6" t="inlineStr">
         <is>
-          <t>As an on-call engineer, I want error tracking and alerting layered on top of the existing metrics, so that I find out about a production problem from a page, not from a driver's phone call.</t>
+          <t>As a hub dispatcher, I want the SLA hold-window minutes recalibrated from real Hub 1 data, so that orders are held just long enough to batch efficiently without risking an SLA breach.</t>
         </is>
       </c>
     </row>
     <row r="27">
       <c r="A27" s="7" t="inlineStr">
         <is>
-          <t>S5</t>
+          <t>E6</t>
         </is>
       </c>
       <c r="B27" s="8" t="inlineStr">
         <is>
-          <t>Security</t>
+          <t>Core backend</t>
         </is>
       </c>
       <c r="C27" s="8" t="inlineStr">
         <is>
-          <t>General API rate limiting</t>
-        </is>
-      </c>
-      <c r="D27" s="9" t="inlineStr">
-        <is>
-          <t>Done</t>
+          <t>Confirm Learning Loop flag-type naming convention</t>
+        </is>
+      </c>
+      <c r="D27" s="7" t="inlineStr">
+        <is>
+          <t>Open</t>
         </is>
       </c>
       <c r="E27" s="8" t="inlineStr">
         <is>
-          <t>Phase 5</t>
+          <t>Phase 4</t>
         </is>
       </c>
       <c r="F27" s="8" t="inlineStr">
         <is>
-          <t>As the platform, I want a per-IP rate limit across the whole API, so that abusive traffic or credential-guessing can't overwhelm the system before authentication even runs.</t>
+          <t>As the engineer building the annotation loop, I want the flag-type naming convention signed off by a driver-app stakeholder, so that the contract between driver annotations and the Learning Loop isn't just an internal guess.</t>
         </is>
       </c>
     </row>
     <row r="28">
       <c r="A28" s="5" t="inlineStr">
         <is>
-          <t>S6</t>
+          <t>E7</t>
         </is>
       </c>
       <c r="B28" s="6" t="inlineStr">
         <is>
-          <t>Security</t>
+          <t>Core backend</t>
         </is>
       </c>
       <c r="C28" s="6" t="inlineStr">
         <is>
-          <t>A real security review</t>
-        </is>
-      </c>
-      <c r="D28" s="5" t="inlineStr">
-        <is>
-          <t>Open</t>
+          <t>Wire a real scheduler for the Learning Loop's nightly job</t>
+        </is>
+      </c>
+      <c r="D28" s="10" t="inlineStr">
+        <is>
+          <t>Done</t>
         </is>
       </c>
       <c r="E28" s="6" t="inlineStr">
         <is>
-          <t>Phase 5</t>
+          <t>Phase 4</t>
         </is>
       </c>
       <c r="F28" s="6" t="inlineStr">
         <is>
-          <t>As LMX leadership, I want an outside security review of the platform, so that real orders, drivers, and eventually payments aren't the first real test of its defenses.</t>
+          <t>As a hub, I want the Learning Loop's nightly detection job to run automatically on schedule, so that rule proposals get generated every night without anyone manually triggering it.</t>
         </is>
       </c>
     </row>
     <row r="29">
       <c r="A29" s="7" t="inlineStr">
         <is>
-          <t>S7</t>
+          <t>E8</t>
         </is>
       </c>
       <c r="B29" s="8" t="inlineStr">
         <is>
-          <t>Security</t>
+          <t>Core backend</t>
         </is>
       </c>
       <c r="C29" s="8" t="inlineStr">
         <is>
-          <t>Twilio inbound-webhook signature verification</t>
+          <t>Move the event bus off in-process</t>
         </is>
       </c>
       <c r="D29" s="9" t="inlineStr">
@@ -1555,88 +1555,88 @@
       </c>
       <c r="F29" s="8" t="inlineStr">
         <is>
-          <t>As the platform receiving inbound SMS webhooks, I want Twilio's signature verified on every request, so that a forged webhook can't inject fake driver replies into the system.</t>
+          <t>As the platform running on more than one instance, I want the event bus backed by Redis instead of in-process memory, so that hold-release and dispatch events stay consistent across multiple app instances.</t>
         </is>
       </c>
     </row>
     <row r="30">
       <c r="A30" s="5" t="inlineStr">
         <is>
-          <t>S8</t>
+          <t>E9</t>
         </is>
       </c>
       <c r="B30" s="6" t="inlineStr">
         <is>
-          <t>Security</t>
+          <t>Core backend</t>
         </is>
       </c>
       <c r="C30" s="6" t="inlineStr">
         <is>
-          <t>Rate-limit client login</t>
-        </is>
-      </c>
-      <c r="D30" s="10" t="inlineStr">
-        <is>
-          <t>Done</t>
+          <t>Validate the 2.5 DPH figure</t>
+        </is>
+      </c>
+      <c r="D30" s="5" t="inlineStr">
+        <is>
+          <t>Open</t>
         </is>
       </c>
       <c r="E30" s="6" t="inlineStr">
         <is>
-          <t>Phase 5</t>
+          <t>Phase 9 (needs B2)</t>
         </is>
       </c>
       <c r="F30" s="6" t="inlineStr">
         <is>
-          <t>As a client company logging into the portal, I want login attempts rate-limited, so that someone else can't brute-force my company's portal password.</t>
+          <t>As LMX leadership, I want the 2.5 deliveries-per-hour assumption validated against real Hub 1 data, so that pricing and staffing decisions rest on a proven number instead of a model assumption.</t>
         </is>
       </c>
     </row>
     <row r="31">
       <c r="A31" s="7" t="inlineStr">
         <is>
-          <t>S9</t>
+          <t>E10</t>
         </is>
       </c>
       <c r="B31" s="8" t="inlineStr">
         <is>
-          <t>Security</t>
+          <t>Core backend</t>
         </is>
       </c>
       <c r="C31" s="8" t="inlineStr">
         <is>
-          <t>Enforce distinct client/driver JWT secrets at startup</t>
-        </is>
-      </c>
-      <c r="D31" s="9" t="inlineStr">
-        <is>
-          <t>Done</t>
+          <t>Tune HOT_SHOT's skip-penalty/hold-window placeholders</t>
+        </is>
+      </c>
+      <c r="D31" s="7" t="inlineStr">
+        <is>
+          <t>Open</t>
         </is>
       </c>
       <c r="E31" s="8" t="inlineStr">
         <is>
-          <t>Phase 5</t>
+          <t>Phase 8 follow-up / I5</t>
         </is>
       </c>
       <c r="F31" s="8" t="inlineStr">
         <is>
-          <t>As the platform, I want the client and driver JWT secrets to be provably different at startup, so that a token issued for one audience can never be replayed as if it were the other.</t>
+          <t>As a hub dispatcher, I want HOT_SHOT's skip-penalty and hold-window values calibrated like the other tiers, so that the premium tier's priority handling is based on real economics, not a guess.</t>
         </is>
       </c>
     </row>
     <row r="32">
       <c r="A32" s="5" t="inlineStr">
         <is>
-          <t>D1</t>
+          <t>S1</t>
         </is>
       </c>
       <c r="B32" s="6" t="inlineStr">
         <is>
-          <t>Ops dashboard</t>
+          <t>Security</t>
         </is>
       </c>
       <c r="C32" s="6" t="inlineStr">
         <is>
-          <t>Add a list-hubs endpoint</t>
+          <t>Real per-user authentication for the ops dashboard</t>
         </is>
       </c>
       <c r="D32" s="10" t="inlineStr">
@@ -1646,61 +1646,61 @@
       </c>
       <c r="E32" s="6" t="inlineStr">
         <is>
-          <t>-</t>
+          <t>Phase 5</t>
         </is>
       </c>
       <c r="F32" s="6" t="inlineStr">
         <is>
-          <t>As a hub ops staff member, I want to pick my hub from a real dropdown instead of typing a UUID, so that I can't accidentally point the dashboard at the wrong hub.</t>
+          <t>As a hub ops manager, I want each staff member to log in with their own account and role, so that I know who did what in the dashboard and can limit admin actions to admins.</t>
         </is>
       </c>
     </row>
     <row r="33">
       <c r="A33" s="7" t="inlineStr">
         <is>
-          <t>D2</t>
+          <t>S2</t>
         </is>
       </c>
       <c r="B33" s="8" t="inlineStr">
         <is>
-          <t>Ops dashboard</t>
+          <t>Security</t>
         </is>
       </c>
       <c r="C33" s="8" t="inlineStr">
         <is>
-          <t>Stop baking the API URL in at Docker build time</t>
-        </is>
-      </c>
-      <c r="D33" s="9" t="inlineStr">
-        <is>
-          <t>Done</t>
+          <t>Secrets management</t>
+        </is>
+      </c>
+      <c r="D33" s="7" t="inlineStr">
+        <is>
+          <t>Open</t>
         </is>
       </c>
       <c r="E33" s="8" t="inlineStr">
         <is>
-          <t>-</t>
+          <t>Phase 5</t>
         </is>
       </c>
       <c r="F33" s="8" t="inlineStr">
         <is>
-          <t>As the engineer deploying the dashboard, I want the API URL configured at container start instead of baked in at build time, so that one built image can point at any environment without a rebuild.</t>
+          <t>As the engineering team, I want credentials stored in a real secrets manager instead of a .env file, so that a leaked file or repo doesn't hand over database passwords and API keys.</t>
         </is>
       </c>
     </row>
     <row r="34">
       <c r="A34" s="5" t="inlineStr">
         <is>
-          <t>A1</t>
+          <t>S3</t>
         </is>
       </c>
       <c r="B34" s="6" t="inlineStr">
         <is>
-          <t>Driver app</t>
+          <t>Security</t>
         </is>
       </c>
       <c r="C34" s="6" t="inlineStr">
         <is>
-          <t>Push notifications</t>
+          <t>A real production hosting decision</t>
         </is>
       </c>
       <c r="D34" s="5" t="inlineStr">
@@ -1710,93 +1710,93 @@
       </c>
       <c r="E34" s="6" t="inlineStr">
         <is>
-          <t>Phase 6</t>
+          <t>Phase 5</t>
         </is>
       </c>
       <c r="F34" s="6" t="inlineStr">
         <is>
-          <t>As a driver, I want a push notification the moment a new job is offered to me, so that I don't have to keep the app open and polling to catch new work.</t>
+          <t>As the engineering team preparing for Hub 1, I want a resilient hosting setup instead of a single-instance docker-compose, so that a container crash or server failure doesn't take down dispatch for real drivers and orders.</t>
         </is>
       </c>
     </row>
     <row r="35">
       <c r="A35" s="7" t="inlineStr">
         <is>
-          <t>A2</t>
+          <t>S4</t>
         </is>
       </c>
       <c r="B35" s="8" t="inlineStr">
         <is>
-          <t>Driver app</t>
+          <t>Security</t>
         </is>
       </c>
       <c r="C35" s="8" t="inlineStr">
         <is>
-          <t>Real camera/barcode scanning</t>
-        </is>
-      </c>
-      <c r="D35" s="7" t="inlineStr">
-        <is>
-          <t>Open</t>
+          <t>Observability</t>
+        </is>
+      </c>
+      <c r="D35" s="11" t="inlineStr">
+        <is>
+          <t>Partial</t>
         </is>
       </c>
       <c r="E35" s="8" t="inlineStr">
         <is>
-          <t>Phase 6</t>
+          <t>Phase 5</t>
         </is>
       </c>
       <c r="F35" s="8" t="inlineStr">
         <is>
-          <t>As a driver scanning parcels at pickup, I want to scan a real barcode, so that the parcel count is accurate instead of a manual tap anyone could get wrong or fake.</t>
+          <t>As an on-call engineer, I want error tracking and alerting layered on top of the existing metrics, so that I find out about a production problem from a page, not from a driver's phone call.</t>
         </is>
       </c>
     </row>
     <row r="36">
       <c r="A36" s="5" t="inlineStr">
         <is>
-          <t>A3</t>
+          <t>S5</t>
         </is>
       </c>
       <c r="B36" s="6" t="inlineStr">
         <is>
-          <t>Driver app</t>
+          <t>Security</t>
         </is>
       </c>
       <c r="C36" s="6" t="inlineStr">
         <is>
-          <t>Real photo/signature capture + upload pipeline</t>
-        </is>
-      </c>
-      <c r="D36" s="5" t="inlineStr">
-        <is>
-          <t>Open</t>
+          <t>General API rate limiting</t>
+        </is>
+      </c>
+      <c r="D36" s="10" t="inlineStr">
+        <is>
+          <t>Done</t>
         </is>
       </c>
       <c r="E36" s="6" t="inlineStr">
         <is>
-          <t>Phase 6</t>
+          <t>Phase 5</t>
         </is>
       </c>
       <c r="F36" s="6" t="inlineStr">
         <is>
-          <t>As a driver completing a delivery, I want to actually capture and upload a photo or signature, so that proof of delivery is a real image on file, not a placeholder URL.</t>
+          <t>As the platform, I want a per-IP rate limit across the whole API, so that abusive traffic or credential-guessing can't overwhelm the system before authentication even runs.</t>
         </is>
       </c>
     </row>
     <row r="37">
       <c r="A37" s="7" t="inlineStr">
         <is>
-          <t>A4</t>
+          <t>S6</t>
         </is>
       </c>
       <c r="B37" s="8" t="inlineStr">
         <is>
-          <t>Driver app</t>
+          <t>Security</t>
         </is>
       </c>
       <c r="C37" s="8" t="inlineStr">
         <is>
-          <t>A real PIN-issuance/verification system</t>
+          <t>A real security review</t>
         </is>
       </c>
       <c r="D37" s="7" t="inlineStr">
@@ -1806,125 +1806,125 @@
       </c>
       <c r="E37" s="8" t="inlineStr">
         <is>
-          <t>Phase 6</t>
+          <t>Phase 5</t>
         </is>
       </c>
       <c r="F37" s="8" t="inlineStr">
         <is>
-          <t>As a driver delivering an order that requires a PIN, I want the PIN checked against a real system, so that I can be confident the person receiving the package is who they say they are.</t>
+          <t>As LMX leadership, I want an outside security review of the platform, so that real orders, drivers, and eventually payments aren't the first real test of its defenses.</t>
         </is>
       </c>
     </row>
     <row r="38">
       <c r="A38" s="5" t="inlineStr">
         <is>
-          <t>A5</t>
+          <t>S7</t>
         </is>
       </c>
       <c r="B38" s="6" t="inlineStr">
         <is>
-          <t>Driver app</t>
+          <t>Security</t>
         </is>
       </c>
       <c r="C38" s="6" t="inlineStr">
         <is>
-          <t>Maps SDK / turn-by-turn navigation</t>
-        </is>
-      </c>
-      <c r="D38" s="5" t="inlineStr">
-        <is>
-          <t>Open</t>
+          <t>Twilio inbound-webhook signature verification</t>
+        </is>
+      </c>
+      <c r="D38" s="10" t="inlineStr">
+        <is>
+          <t>Done</t>
         </is>
       </c>
       <c r="E38" s="6" t="inlineStr">
         <is>
-          <t>Phase 6</t>
+          <t>Phase 5</t>
         </is>
       </c>
       <c r="F38" s="6" t="inlineStr">
         <is>
-          <t>As a driver on route, I want live turn-by-turn navigation in the app, so that I don't need a separate maps app to find each stop.</t>
+          <t>As the platform receiving inbound SMS webhooks, I want Twilio's signature verified on every request, so that a forged webhook can't inject fake driver replies into the system.</t>
         </is>
       </c>
     </row>
     <row r="39">
       <c r="A39" s="7" t="inlineStr">
         <is>
-          <t>A6</t>
+          <t>S8</t>
         </is>
       </c>
       <c r="B39" s="8" t="inlineStr">
         <is>
-          <t>Driver app</t>
+          <t>Security</t>
         </is>
       </c>
       <c r="C39" s="8" t="inlineStr">
         <is>
-          <t>Mobile app store deployment pipeline</t>
-        </is>
-      </c>
-      <c r="D39" s="7" t="inlineStr">
-        <is>
-          <t>Open</t>
+          <t>Rate-limit client login</t>
+        </is>
+      </c>
+      <c r="D39" s="9" t="inlineStr">
+        <is>
+          <t>Done</t>
         </is>
       </c>
       <c r="E39" s="8" t="inlineStr">
         <is>
-          <t>Phase 6</t>
+          <t>Phase 5</t>
         </is>
       </c>
       <c r="F39" s="8" t="inlineStr">
         <is>
-          <t>As a driver, I want to install the app from TestFlight or the Play Store, so that I don't need developer tooling just to get the app on my phone.</t>
+          <t>As a client company logging into the portal, I want login attempts rate-limited, so that someone else can't brute-force my company's portal password.</t>
         </is>
       </c>
     </row>
     <row r="40">
       <c r="A40" s="5" t="inlineStr">
         <is>
-          <t>A7</t>
+          <t>S9</t>
         </is>
       </c>
       <c r="B40" s="6" t="inlineStr">
         <is>
-          <t>Driver app</t>
+          <t>Security</t>
         </is>
       </c>
       <c r="C40" s="6" t="inlineStr">
         <is>
-          <t>Masked voice calling</t>
-        </is>
-      </c>
-      <c r="D40" s="5" t="inlineStr">
-        <is>
-          <t>Open</t>
+          <t>Enforce distinct client/driver JWT secrets at startup</t>
+        </is>
+      </c>
+      <c r="D40" s="10" t="inlineStr">
+        <is>
+          <t>Done</t>
         </is>
       </c>
       <c r="E40" s="6" t="inlineStr">
         <is>
-          <t>Phase 6</t>
+          <t>Phase 5</t>
         </is>
       </c>
       <c r="F40" s="6" t="inlineStr">
         <is>
-          <t>As a driver or customer who needs to talk instead of text, I want a masked voice call option, so that we can resolve an issue quickly without exposing either party's real phone number.</t>
+          <t>As the platform, I want the client and driver JWT secrets to be provably different at startup, so that a token issued for one audience can never be replayed as if it were the other.</t>
         </is>
       </c>
     </row>
     <row r="41">
       <c r="A41" s="7" t="inlineStr">
         <is>
-          <t>A8</t>
+          <t>D1</t>
         </is>
       </c>
       <c r="B41" s="8" t="inlineStr">
         <is>
-          <t>Driver app</t>
+          <t>Ops dashboard</t>
         </is>
       </c>
       <c r="C41" s="8" t="inlineStr">
         <is>
-          <t>Harden inbound-SMS reply matching</t>
+          <t>Add a list-hubs endpoint</t>
         </is>
       </c>
       <c r="D41" s="9" t="inlineStr">
@@ -1934,221 +1934,221 @@
       </c>
       <c r="E41" s="8" t="inlineStr">
         <is>
-          <t>Phase 6</t>
+          <t>-</t>
         </is>
       </c>
       <c r="F41" s="8" t="inlineStr">
         <is>
-          <t>As a shop replying to a delivery SMS, I want my reply matched to the correct, active conversation, so that my message doesn't get attached to the wrong or already-completed stop.</t>
+          <t>As a hub ops staff member, I want to pick my hub from a real dropdown instead of typing a UUID, so that I can't accidentally point the dashboard at the wrong hub.</t>
         </is>
       </c>
     </row>
     <row r="42">
       <c r="A42" s="5" t="inlineStr">
         <is>
-          <t>A9</t>
+          <t>D2</t>
         </is>
       </c>
       <c r="B42" s="6" t="inlineStr">
         <is>
-          <t>Driver app</t>
+          <t>Ops dashboard</t>
         </is>
       </c>
       <c r="C42" s="6" t="inlineStr">
         <is>
-          <t>Real earnings formula + payroll integration</t>
-        </is>
-      </c>
-      <c r="D42" s="11" t="inlineStr">
-        <is>
-          <t>Partial (scaffolding shipped)</t>
+          <t>Stop baking the API URL in at Docker build time</t>
+        </is>
+      </c>
+      <c r="D42" s="10" t="inlineStr">
+        <is>
+          <t>Done</t>
         </is>
       </c>
       <c r="E42" s="6" t="inlineStr">
         <is>
-          <t>Phase 7</t>
+          <t>-</t>
         </is>
       </c>
       <c r="F42" s="6" t="inlineStr">
         <is>
-          <t>As a driver, I want my earnings screen to show a real, calculated number tied to actual payroll, so that I know what I'll actually be paid instead of seeing a placeholder.</t>
+          <t>As the engineer deploying the dashboard, I want the API URL configured at container start instead of baked in at build time, so that one built image can point at any environment without a rebuild.</t>
         </is>
       </c>
     </row>
     <row r="43">
       <c r="A43" s="7" t="inlineStr">
         <is>
-          <t>C1</t>
+          <t>A1</t>
         </is>
       </c>
       <c r="B43" s="8" t="inlineStr">
         <is>
-          <t>Components</t>
+          <t>Driver app</t>
         </is>
       </c>
       <c r="C43" s="8" t="inlineStr">
         <is>
-          <t>Client-facing dashboard</t>
-        </is>
-      </c>
-      <c r="D43" s="9" t="inlineStr">
-        <is>
-          <t>Done (Phase 8)</t>
+          <t>Push notifications</t>
+        </is>
+      </c>
+      <c r="D43" s="7" t="inlineStr">
+        <is>
+          <t>Open</t>
         </is>
       </c>
       <c r="E43" s="8" t="inlineStr">
         <is>
-          <t>-</t>
+          <t>Phase 6</t>
         </is>
       </c>
       <c r="F43" s="8" t="inlineStr">
         <is>
-          <t>As a client company, I want a portal showing my order history, status, and fees, so that I don't have to call LMX to know where my orders stand.</t>
+          <t>As a driver, I want a push notification the moment a new job is offered to me, so that I don't have to keep the app open and polling to catch new work.</t>
         </is>
       </c>
     </row>
     <row r="44">
       <c r="A44" s="5" t="inlineStr">
         <is>
-          <t>C2</t>
+          <t>A2</t>
         </is>
       </c>
       <c r="B44" s="6" t="inlineStr">
         <is>
-          <t>Components</t>
+          <t>Driver app</t>
         </is>
       </c>
       <c r="C44" s="6" t="inlineStr">
         <is>
-          <t>Shop SMS</t>
-        </is>
-      </c>
-      <c r="D44" s="10" t="inlineStr">
-        <is>
-          <t>Done (Phase 8)</t>
+          <t>Real camera/barcode scanning</t>
+        </is>
+      </c>
+      <c r="D44" s="5" t="inlineStr">
+        <is>
+          <t>Open</t>
         </is>
       </c>
       <c r="E44" s="6" t="inlineStr">
         <is>
-          <t>-</t>
+          <t>Phase 6</t>
         </is>
       </c>
       <c r="F44" s="6" t="inlineStr">
         <is>
-          <t>As a shop, I want an automatic text when my order is picked up and when the driver's en route, so that I don't have to guess or call in to check.</t>
+          <t>As a driver scanning parcels at pickup, I want to scan a real barcode, so that the parcel count is accurate instead of a manual tap anyone could get wrong or fake.</t>
         </is>
       </c>
     </row>
     <row r="45">
       <c r="A45" s="7" t="inlineStr">
         <is>
-          <t>C3</t>
+          <t>A3</t>
         </is>
       </c>
       <c r="B45" s="8" t="inlineStr">
         <is>
-          <t>Components</t>
+          <t>Driver app</t>
         </is>
       </c>
       <c r="C45" s="8" t="inlineStr">
         <is>
-          <t>A real billing/invoicing system</t>
-        </is>
-      </c>
-      <c r="D45" s="12" t="inlineStr">
-        <is>
-          <t>Partial</t>
+          <t>Real photo/signature capture + upload pipeline</t>
+        </is>
+      </c>
+      <c r="D45" s="7" t="inlineStr">
+        <is>
+          <t>Open</t>
         </is>
       </c>
       <c r="E45" s="8" t="inlineStr">
         <is>
-          <t>Phase 8 follow-up</t>
+          <t>Phase 6</t>
         </is>
       </c>
       <c r="F45" s="8" t="inlineStr">
         <is>
-          <t>As a client company, I want a real monthly statement and invoice I can download, so that I can reconcile what I owe LMX without manually recomputing it from order history.</t>
+          <t>As a driver completing a delivery, I want to actually capture and upload a photo or signature, so that proof of delivery is a real image on file, not a placeholder URL.</t>
         </is>
       </c>
     </row>
     <row r="46">
       <c r="A46" s="5" t="inlineStr">
         <is>
-          <t>C4</t>
+          <t>A4</t>
         </is>
       </c>
       <c r="B46" s="6" t="inlineStr">
         <is>
-          <t>Components</t>
+          <t>Driver app</t>
         </is>
       </c>
       <c r="C46" s="6" t="inlineStr">
         <is>
-          <t>Multi-user client accounts</t>
+          <t>A real PIN-issuance/verification system</t>
         </is>
       </c>
       <c r="D46" s="5" t="inlineStr">
         <is>
-          <t>Open (deliberate, later)</t>
+          <t>Open</t>
         </is>
       </c>
       <c r="E46" s="6" t="inlineStr">
         <is>
-          <t>Phase 8 follow-up</t>
+          <t>Phase 6</t>
         </is>
       </c>
       <c r="F46" s="6" t="inlineStr">
         <is>
-          <t>As a client company with both an AP contact and an ops contact, I want more than one login for my company, so that each person can access the portal without sharing one password.</t>
+          <t>As a driver delivering an order that requires a PIN, I want the PIN checked against a real system, so that I can be confident the person receiving the package is who they say they are.</t>
         </is>
       </c>
     </row>
     <row r="47">
       <c r="A47" s="7" t="inlineStr">
         <is>
-          <t>C5</t>
+          <t>A5</t>
         </is>
       </c>
       <c r="B47" s="8" t="inlineStr">
         <is>
-          <t>Components</t>
+          <t>Driver app</t>
         </is>
       </c>
       <c r="C47" s="8" t="inlineStr">
         <is>
-          <t>Self-service client signup</t>
-        </is>
-      </c>
-      <c r="D47" s="13" t="inlineStr">
-        <is>
-          <t>Deliberately not building</t>
+          <t>Maps SDK / turn-by-turn navigation</t>
+        </is>
+      </c>
+      <c r="D47" s="7" t="inlineStr">
+        <is>
+          <t>Open</t>
         </is>
       </c>
       <c r="E47" s="8" t="inlineStr">
         <is>
-          <t>-</t>
+          <t>Phase 6</t>
         </is>
       </c>
       <c r="F47" s="8" t="inlineStr">
         <is>
-          <t>As LMX's business development team, we deliberately do not want a self-serve client signup flow, so that every new client relationship stays a real onboarding conversation, matching a B2B operator model rather than self-serve SaaS.</t>
+          <t>As a driver on route, I want live turn-by-turn navigation in the app, so that I don't need a separate maps app to find each stop.</t>
         </is>
       </c>
     </row>
     <row r="48">
       <c r="A48" s="5" t="inlineStr">
         <is>
-          <t>P1</t>
+          <t>A6</t>
         </is>
       </c>
       <c r="B48" s="6" t="inlineStr">
         <is>
-          <t>Autonomy partners</t>
+          <t>Driver app</t>
         </is>
       </c>
       <c r="C48" s="6" t="inlineStr">
         <is>
-          <t>Courier abstraction over the fleet model</t>
+          <t>Mobile app store deployment pipeline</t>
         </is>
       </c>
       <c r="D48" s="5" t="inlineStr">
@@ -2158,29 +2158,29 @@
       </c>
       <c r="E48" s="6" t="inlineStr">
         <is>
-          <t>Phase 11 (Track A gate)</t>
+          <t>Phase 6</t>
         </is>
       </c>
       <c r="F48" s="6" t="inlineStr">
         <is>
-          <t>As the engineering team, I want the fleet model generalized into a courier abstraction (human driver, autonomy partner, or gig courier), so that adding a new capacity type later doesn't require reworking code that assumes every courier is a person.</t>
+          <t>As a driver, I want to install the app from TestFlight or the Play Store, so that I don't need developer tooling just to get the app on my phone.</t>
         </is>
       </c>
     </row>
     <row r="49">
       <c r="A49" s="7" t="inlineStr">
         <is>
-          <t>P2</t>
+          <t>A7</t>
         </is>
       </c>
       <c r="B49" s="8" t="inlineStr">
         <is>
-          <t>Autonomy partners</t>
+          <t>Driver app</t>
         </is>
       </c>
       <c r="C49" s="8" t="inlineStr">
         <is>
-          <t>Capacity-provider adapter layer</t>
+          <t>Masked voice calling</t>
         </is>
       </c>
       <c r="D49" s="7" t="inlineStr">
@@ -2190,253 +2190,253 @@
       </c>
       <c r="E49" s="8" t="inlineStr">
         <is>
-          <t>Phase 11 (Track A gate)</t>
+          <t>Phase 6</t>
         </is>
       </c>
       <c r="F49" s="8" t="inlineStr">
         <is>
-          <t>As the engineering team, I want one adapter per capacity partner normalizing capacity, assignment, and status, so that onboarding a new autonomy or gig partner doesn't mean writing bespoke dispatch logic each time.</t>
+          <t>As a driver or customer who needs to talk instead of text, I want a masked voice call option, so that we can resolve an issue quickly without exposing either party's real phone number.</t>
         </is>
       </c>
     </row>
     <row r="50">
       <c r="A50" s="5" t="inlineStr">
         <is>
-          <t>P3</t>
+          <t>A8</t>
         </is>
       </c>
       <c r="B50" s="6" t="inlineStr">
         <is>
-          <t>Autonomy partners</t>
+          <t>Driver app</t>
         </is>
       </c>
       <c r="C50" s="6" t="inlineStr">
         <is>
-          <t>Mode-aware dispatch</t>
-        </is>
-      </c>
-      <c r="D50" s="5" t="inlineStr">
-        <is>
-          <t>Open</t>
+          <t>Harden inbound-SMS reply matching</t>
+        </is>
+      </c>
+      <c r="D50" s="10" t="inlineStr">
+        <is>
+          <t>Done</t>
         </is>
       </c>
       <c r="E50" s="6" t="inlineStr">
         <is>
-          <t>Phase 11</t>
+          <t>Phase 6</t>
         </is>
       </c>
       <c r="F50" s="6" t="inlineStr">
         <is>
-          <t>As a hub dispatcher, I want the optimizer to filter and choose the cheapest eligible delivery mode per order, so that a 40lb order never gets offered to a bike courier and cost-per-drop stays optimized across every available mode.</t>
+          <t>As a shop replying to a delivery SMS, I want my reply matched to the correct, active conversation, so that my message doesn't get attached to the wrong or already-completed stop.</t>
         </is>
       </c>
     </row>
     <row r="51">
       <c r="A51" s="7" t="inlineStr">
         <is>
-          <t>P4</t>
+          <t>A9</t>
         </is>
       </c>
       <c r="B51" s="8" t="inlineStr">
         <is>
-          <t>Autonomy partners</t>
+          <t>Driver app</t>
         </is>
       </c>
       <c r="C51" s="8" t="inlineStr">
         <is>
-          <t>Unmanned handoff + proof of delivery</t>
-        </is>
-      </c>
-      <c r="D51" s="7" t="inlineStr">
-        <is>
-          <t>Open</t>
+          <t>Real earnings formula + payroll integration</t>
+        </is>
+      </c>
+      <c r="D51" s="11" t="inlineStr">
+        <is>
+          <t>Partial (scaffolding shipped)</t>
         </is>
       </c>
       <c r="E51" s="8" t="inlineStr">
         <is>
-          <t>Phase 11 (shares A4)</t>
+          <t>Phase 7</t>
         </is>
       </c>
       <c r="F51" s="8" t="inlineStr">
         <is>
-          <t>As a shop receiving an autonomous vehicle for pickup, I want a clear load-confirmation flow, so that handing off a parcel to a bot is as unambiguous as handing it to a driver.</t>
+          <t>As a driver, I want my earnings screen to show a real, calculated number tied to actual payroll, so that I know what I'll actually be paid instead of seeing a placeholder.</t>
         </is>
       </c>
     </row>
     <row r="52">
       <c r="A52" s="5" t="inlineStr">
         <is>
-          <t>P5</t>
+          <t>C1</t>
         </is>
       </c>
       <c r="B52" s="6" t="inlineStr">
         <is>
-          <t>Autonomy partners</t>
+          <t>Components</t>
         </is>
       </c>
       <c r="C52" s="6" t="inlineStr">
         <is>
-          <t>Partner settlement</t>
-        </is>
-      </c>
-      <c r="D52" s="5" t="inlineStr">
-        <is>
-          <t>Open</t>
+          <t>Client-facing dashboard</t>
+        </is>
+      </c>
+      <c r="D52" s="10" t="inlineStr">
+        <is>
+          <t>Done (Phase 8)</t>
         </is>
       </c>
       <c r="E52" s="6" t="inlineStr">
         <is>
-          <t>Phase 11 (later)</t>
+          <t>-</t>
         </is>
       </c>
       <c r="F52" s="6" t="inlineStr">
         <is>
-          <t>As an autonomy or gig-courier partner, I want a monthly settlement statement for the deliveries I carried, so that I get paid accurately without a manual reconciliation with LMX.</t>
+          <t>As a client company, I want a portal showing my order history, status, and fees, so that I don't have to call LMX to know where my orders stand.</t>
         </is>
       </c>
     </row>
     <row r="53">
       <c r="A53" s="7" t="inlineStr">
         <is>
-          <t>P6</t>
+          <t>C2</t>
         </is>
       </c>
       <c r="B53" s="8" t="inlineStr">
         <is>
-          <t>Autonomy partners</t>
+          <t>Components</t>
         </is>
       </c>
       <c r="C53" s="8" t="inlineStr">
         <is>
-          <t>Partner portal</t>
-        </is>
-      </c>
-      <c r="D53" s="7" t="inlineStr">
-        <is>
-          <t>Open</t>
+          <t>Shop SMS</t>
+        </is>
+      </c>
+      <c r="D53" s="9" t="inlineStr">
+        <is>
+          <t>Done (Phase 8)</t>
         </is>
       </c>
       <c r="E53" s="8" t="inlineStr">
         <is>
-          <t>Phase 11 (later)</t>
+          <t>-</t>
         </is>
       </c>
       <c r="F53" s="8" t="inlineStr">
         <is>
-          <t>As an autonomy or gig-courier partner, I want a portal showing my delivery history and settlement statements, so that I can check my own performance and pay without emailing LMX ops.</t>
+          <t>As a shop, I want an automatic text when my order is picked up and when the driver's en route, so that I don't have to guess or call in to check.</t>
         </is>
       </c>
     </row>
     <row r="54">
       <c r="A54" s="5" t="inlineStr">
         <is>
-          <t>P7</t>
+          <t>C3</t>
         </is>
       </c>
       <c r="B54" s="6" t="inlineStr">
         <is>
-          <t>Autonomy partners</t>
+          <t>Components</t>
         </is>
       </c>
       <c r="C54" s="6" t="inlineStr">
         <is>
-          <t>Gig-courier cost-optimized dispatch</t>
-        </is>
-      </c>
-      <c r="D54" s="5" t="inlineStr">
-        <is>
-          <t>Open (gated on unit economics)</t>
+          <t>A real billing/invoicing system</t>
+        </is>
+      </c>
+      <c r="D54" s="12" t="inlineStr">
+        <is>
+          <t>Partial</t>
         </is>
       </c>
       <c r="E54" s="6" t="inlineStr">
         <is>
-          <t>Phase 11 (Track B)</t>
+          <t>Phase 8 follow-up</t>
         </is>
       </c>
       <c r="F54" s="6" t="inlineStr">
         <is>
-          <t>As LMX leadership, I want the option to route an order to a gig courier when it's genuinely the cheaper eligible choice, so that capacity can flex without ever changing the client's brand, SLA, or bill - capped and tagged so it never masks LMX's own unit economics.</t>
+          <t>As a client company, I want a real monthly statement and invoice I can download, so that I can reconcile what I owe LMX without manually recomputing it from order history.</t>
         </is>
       </c>
     </row>
     <row r="55">
       <c r="A55" s="7" t="inlineStr">
         <is>
-          <t>F1</t>
+          <t>C4</t>
         </is>
       </c>
       <c r="B55" s="8" t="inlineStr">
         <is>
-          <t>Competitive gaps</t>
+          <t>Components</t>
         </is>
       </c>
       <c r="C55" s="8" t="inlineStr">
         <is>
-          <t>Live driver location pipeline</t>
+          <t>Multi-user client accounts</t>
         </is>
       </c>
       <c r="D55" s="7" t="inlineStr">
         <is>
-          <t>Open</t>
+          <t>Open (deliberate, later)</t>
         </is>
       </c>
       <c r="E55" s="8" t="inlineStr">
         <is>
-          <t>Phase 6</t>
+          <t>Phase 8 follow-up</t>
         </is>
       </c>
       <c r="F55" s="8" t="inlineStr">
         <is>
-          <t>As the platform, I want the driver app to periodically report its location, so that there's a real, current position on file for every driver on shift.</t>
+          <t>As a client company with both an AP contact and an ops contact, I want more than one login for my company, so that each person can access the portal without sharing one password.</t>
         </is>
       </c>
     </row>
     <row r="56">
       <c r="A56" s="5" t="inlineStr">
         <is>
-          <t>F2</t>
+          <t>C5</t>
         </is>
       </c>
       <c r="B56" s="6" t="inlineStr">
         <is>
-          <t>Competitive gaps</t>
+          <t>Components</t>
         </is>
       </c>
       <c r="C56" s="6" t="inlineStr">
         <is>
-          <t>Live map view (ops dashboard)</t>
-        </is>
-      </c>
-      <c r="D56" s="5" t="inlineStr">
-        <is>
-          <t>Open</t>
+          <t>Self-service client signup</t>
+        </is>
+      </c>
+      <c r="D56" s="13" t="inlineStr">
+        <is>
+          <t>Deliberately not building</t>
         </is>
       </c>
       <c r="E56" s="6" t="inlineStr">
         <is>
-          <t>Phase 6</t>
+          <t>-</t>
         </is>
       </c>
       <c r="F56" s="6" t="inlineStr">
         <is>
-          <t>As a hub ops manager, I want to see every driver's live position on a map, so that I know where my fleet actually is, not just what stop list each driver was assigned.</t>
+          <t>As LMX's business development team, we deliberately do not want a self-serve client signup flow, so that every new client relationship stays a real onboarding conversation, matching a B2B operator model rather than self-serve SaaS.</t>
         </is>
       </c>
     </row>
     <row r="57">
       <c r="A57" s="7" t="inlineStr">
         <is>
-          <t>F3</t>
+          <t>P1</t>
         </is>
       </c>
       <c r="B57" s="8" t="inlineStr">
         <is>
-          <t>Competitive gaps</t>
+          <t>Autonomy partners</t>
         </is>
       </c>
       <c r="C57" s="8" t="inlineStr">
         <is>
-          <t>Customer-facing live tracking page</t>
+          <t>Courier abstraction over the fleet model</t>
         </is>
       </c>
       <c r="D57" s="7" t="inlineStr">
@@ -2446,29 +2446,29 @@
       </c>
       <c r="E57" s="8" t="inlineStr">
         <is>
-          <t>Phase 8 follow-up</t>
+          <t>Phase 11 (Track A gate)</t>
         </is>
       </c>
       <c r="F57" s="8" t="inlineStr">
         <is>
-          <t>As the person receiving a delivery, I want a link that shows my driver's live position and ETA, so that I don't have to call the shop or guess when my part will arrive.</t>
+          <t>As the engineering team, I want the fleet model generalized into a courier abstraction (human driver, autonomy partner, or gig courier), so that adding a new capacity type later doesn't require reworking code that assumes every courier is a person.</t>
         </is>
       </c>
     </row>
     <row r="58">
       <c r="A58" s="5" t="inlineStr">
         <is>
-          <t>F4</t>
+          <t>P2</t>
         </is>
       </c>
       <c r="B58" s="6" t="inlineStr">
         <is>
-          <t>Competitive gaps</t>
+          <t>Autonomy partners</t>
         </is>
       </c>
       <c r="C58" s="6" t="inlineStr">
         <is>
-          <t>Outbound status webhooks + integrations surface</t>
+          <t>Capacity-provider adapter layer</t>
         </is>
       </c>
       <c r="D58" s="5" t="inlineStr">
@@ -2478,29 +2478,29 @@
       </c>
       <c r="E58" s="6" t="inlineStr">
         <is>
-          <t>Phase 8 follow-up</t>
+          <t>Phase 11 (Track A gate)</t>
         </is>
       </c>
       <c r="F58" s="6" t="inlineStr">
         <is>
-          <t>As a client's system administrator, I want to subscribe to order status webhooks, so that my own systems update automatically instead of polling or waiting on a manual check.</t>
+          <t>As the engineering team, I want one adapter per capacity partner normalizing capacity, assignment, and status, so that onboarding a new autonomy or gig partner doesn't mean writing bespoke dispatch logic each time.</t>
         </is>
       </c>
     </row>
     <row r="59">
       <c r="A59" s="7" t="inlineStr">
         <is>
-          <t>F5</t>
+          <t>P3</t>
         </is>
       </c>
       <c r="B59" s="8" t="inlineStr">
         <is>
-          <t>Competitive gaps</t>
+          <t>Autonomy partners</t>
         </is>
       </c>
       <c r="C59" s="8" t="inlineStr">
         <is>
-          <t>Flexible/rate-table billing</t>
+          <t>Mode-aware dispatch</t>
         </is>
       </c>
       <c r="D59" s="7" t="inlineStr">
@@ -2510,29 +2510,29 @@
       </c>
       <c r="E59" s="8" t="inlineStr">
         <is>
-          <t>Phase 8 follow-up</t>
+          <t>Phase 11</t>
         </is>
       </c>
       <c r="F59" s="8" t="inlineStr">
         <is>
-          <t>As a client with orders of very different sizes, I want billing that can reflect piece count, weight, or mileage, not just a flat per-drop rate, so that pricing matches the actual cost of serving my orders.</t>
+          <t>As a hub dispatcher, I want the optimizer to filter and choose the cheapest eligible delivery mode per order, so that a 40lb order never gets offered to a bike courier and cost-per-drop stays optimized across every available mode.</t>
         </is>
       </c>
     </row>
     <row r="60">
       <c r="A60" s="5" t="inlineStr">
         <is>
-          <t>F6</t>
+          <t>P4</t>
         </is>
       </c>
       <c r="B60" s="6" t="inlineStr">
         <is>
-          <t>Competitive gaps</t>
+          <t>Autonomy partners</t>
         </is>
       </c>
       <c r="C60" s="6" t="inlineStr">
         <is>
-          <t>Real-time mid-route re-optimization</t>
+          <t>Unmanned handoff + proof of delivery</t>
         </is>
       </c>
       <c r="D60" s="5" t="inlineStr">
@@ -2542,29 +2542,29 @@
       </c>
       <c r="E60" s="6" t="inlineStr">
         <is>
-          <t>Phase 4 (needs E1)</t>
+          <t>Phase 11 (shares A4)</t>
         </is>
       </c>
       <c r="F60" s="6" t="inlineStr">
         <is>
-          <t>As a hub dispatcher, I want the optimizer to re-sequence an in-progress route when conditions change, so that a driver isn't stuck following a plan that's gone stale since the last cycle.</t>
+          <t>As a shop receiving an autonomous vehicle for pickup, I want a clear load-confirmation flow, so that handing off a parcel to a bot is as unambiguous as handing it to a driver.</t>
         </is>
       </c>
     </row>
     <row r="61">
       <c r="A61" s="7" t="inlineStr">
         <is>
-          <t>F7</t>
+          <t>P5</t>
         </is>
       </c>
       <c r="B61" s="8" t="inlineStr">
         <is>
-          <t>Competitive gaps</t>
+          <t>Autonomy partners</t>
         </is>
       </c>
       <c r="C61" s="8" t="inlineStr">
         <is>
-          <t>Client- and ops-facing analytics dashboards</t>
+          <t>Partner settlement</t>
         </is>
       </c>
       <c r="D61" s="7" t="inlineStr">
@@ -2574,29 +2574,29 @@
       </c>
       <c r="E61" s="8" t="inlineStr">
         <is>
-          <t>Phase 10 (folds into I4)</t>
+          <t>Phase 11 (later)</t>
         </is>
       </c>
       <c r="F61" s="8" t="inlineStr">
         <is>
-          <t>As a client company, I want to see my own on-time rate, volume, and cost trend in the portal, so that I have concrete proof of the value of switching to per-drop pricing with LMX.</t>
+          <t>As an autonomy or gig-courier partner, I want a monthly settlement statement for the deliveries I carried, so that I get paid accurately without a manual reconciliation with LMX.</t>
         </is>
       </c>
     </row>
     <row r="62">
       <c r="A62" s="5" t="inlineStr">
         <is>
-          <t>F8</t>
+          <t>P6</t>
         </is>
       </c>
       <c r="B62" s="6" t="inlineStr">
         <is>
-          <t>Competitive gaps</t>
+          <t>Autonomy partners</t>
         </is>
       </c>
       <c r="C62" s="6" t="inlineStr">
         <is>
-          <t>White-label / multi-brand portal theming</t>
+          <t>Partner portal</t>
         </is>
       </c>
       <c r="D62" s="5" t="inlineStr">
@@ -2606,51 +2606,51 @@
       </c>
       <c r="E62" s="6" t="inlineStr">
         <is>
-          <t>Phase 8 follow-up</t>
+          <t>Phase 11 (later)</t>
         </is>
       </c>
       <c r="F62" s="6" t="inlineStr">
         <is>
-          <t>As a reselling partner, I want the client portal to carry my own brand, so that my customers experience it as part of my business, not a visibly third-party tool.</t>
+          <t>As an autonomy or gig-courier partner, I want a portal showing my delivery history and settlement statements, so that I can check my own performance and pay without emailing LMX ops.</t>
         </is>
       </c>
     </row>
     <row r="63">
       <c r="A63" s="7" t="inlineStr">
         <is>
-          <t>F9</t>
+          <t>P7</t>
         </is>
       </c>
       <c r="B63" s="8" t="inlineStr">
         <is>
-          <t>Competitive gaps</t>
+          <t>Autonomy partners</t>
         </is>
       </c>
       <c r="C63" s="8" t="inlineStr">
         <is>
-          <t>Hybrid gig-fleet overflow dispatch</t>
-        </is>
-      </c>
-      <c r="D63" s="13" t="inlineStr">
-        <is>
-          <t>Superseded -&gt; reinstated as P7</t>
+          <t>Gig-courier cost-optimized dispatch</t>
+        </is>
+      </c>
+      <c r="D63" s="7" t="inlineStr">
+        <is>
+          <t>Open (gated on unit economics)</t>
         </is>
       </c>
       <c r="E63" s="8" t="inlineStr">
         <is>
-          <t>-</t>
+          <t>Phase 11 (Track B)</t>
         </is>
       </c>
       <c r="F63" s="8" t="inlineStr">
         <is>
-          <t>Superseded: see P7 for the current, generalized version of this story (LMX leadership routing to the cheapest eligible capacity, including gig couriers).</t>
+          <t>As LMX leadership, I want the option to route an order to a gig courier when it's genuinely the cheaper eligible choice, so that capacity can flex without ever changing the client's brand, SLA, or bill - capped and tagged so it never masks LMX's own unit economics.</t>
         </is>
       </c>
     </row>
     <row r="64">
       <c r="A64" s="5" t="inlineStr">
         <is>
-          <t>F10</t>
+          <t>F1</t>
         </is>
       </c>
       <c r="B64" s="6" t="inlineStr">
@@ -2660,7 +2660,7 @@
       </c>
       <c r="C64" s="6" t="inlineStr">
         <is>
-          <t>A real path to SOC 2 (or equivalent) certification</t>
+          <t>Live driver location pipeline</t>
         </is>
       </c>
       <c r="D64" s="5" t="inlineStr">
@@ -2670,19 +2670,19 @@
       </c>
       <c r="E64" s="6" t="inlineStr">
         <is>
-          <t>Phase 5</t>
+          <t>Phase 6</t>
         </is>
       </c>
       <c r="F64" s="6" t="inlineStr">
         <is>
-          <t>As an enterprise client's security team, I want to see a SOC 2 report before signing, so that I have independent assurance LMX handles data and access responsibly.</t>
+          <t>As the platform, I want the driver app to periodically report its location, so that there's a real, current position on file for every driver on shift.</t>
         </is>
       </c>
     </row>
     <row r="65">
       <c r="A65" s="7" t="inlineStr">
         <is>
-          <t>F11</t>
+          <t>F2</t>
         </is>
       </c>
       <c r="B65" s="8" t="inlineStr">
@@ -2692,7 +2692,7 @@
       </c>
       <c r="C65" s="8" t="inlineStr">
         <is>
-          <t>SSO/SAML for ops and client logins</t>
+          <t>Live map view (ops dashboard)</t>
         </is>
       </c>
       <c r="D65" s="7" t="inlineStr">
@@ -2702,19 +2702,19 @@
       </c>
       <c r="E65" s="8" t="inlineStr">
         <is>
-          <t>Phase 5</t>
+          <t>Phase 6</t>
         </is>
       </c>
       <c r="F65" s="8" t="inlineStr">
         <is>
-          <t>As an enterprise client's IT admin, I want to enforce SSO for anyone accessing the portal, so that portal access follows the same identity policy as the rest of my company's tools.</t>
+          <t>As a hub ops manager, I want to see every driver's live position on a map, so that I know where my fleet actually is, not just what stop list each driver was assigned.</t>
         </is>
       </c>
     </row>
     <row r="66">
       <c r="A66" s="5" t="inlineStr">
         <is>
-          <t>F12</t>
+          <t>F3</t>
         </is>
       </c>
       <c r="B66" s="6" t="inlineStr">
@@ -2724,7 +2724,7 @@
       </c>
       <c r="C66" s="6" t="inlineStr">
         <is>
-          <t>Network/territory optimization tooling</t>
+          <t>Customer-facing live tracking page</t>
         </is>
       </c>
       <c r="D66" s="5" t="inlineStr">
@@ -2734,19 +2734,19 @@
       </c>
       <c r="E66" s="6" t="inlineStr">
         <is>
-          <t>Later, multi-hub</t>
+          <t>Phase 8 follow-up</t>
         </is>
       </c>
       <c r="F66" s="6" t="inlineStr">
         <is>
-          <t>As LMX leadership planning a second or third hub, I want tooling to redesign depot/zone boundaries, so that expansion decisions are based on a real optimization model instead of intuition.</t>
+          <t>As the person receiving a delivery, I want a link that shows my driver's live position and ETA, so that I don't have to call the shop or guess when my part will arrive.</t>
         </is>
       </c>
     </row>
     <row r="67">
       <c r="A67" s="7" t="inlineStr">
         <is>
-          <t>F13</t>
+          <t>F4</t>
         </is>
       </c>
       <c r="B67" s="8" t="inlineStr">
@@ -2756,7 +2756,7 @@
       </c>
       <c r="C67" s="8" t="inlineStr">
         <is>
-          <t>Ratings &amp; feedback capture</t>
+          <t>Outbound status webhooks + integrations surface</t>
         </is>
       </c>
       <c r="D67" s="7" t="inlineStr">
@@ -2771,14 +2771,14 @@
       </c>
       <c r="F67" s="8" t="inlineStr">
         <is>
-          <t>As a shop after a delivery, I want to leave a quick rating and comment, so that LMX knows how the delivery actually went, not just whether the status says completed.</t>
+          <t>As a client's system administrator, I want to subscribe to order status webhooks, so that my own systems update automatically instead of polling or waiting on a manual check.</t>
         </is>
       </c>
     </row>
     <row r="68">
       <c r="A68" s="5" t="inlineStr">
         <is>
-          <t>F14</t>
+          <t>F5</t>
         </is>
       </c>
       <c r="B68" s="6" t="inlineStr">
@@ -2788,7 +2788,7 @@
       </c>
       <c r="C68" s="6" t="inlineStr">
         <is>
-          <t>Orchestrator route-preview / shadow mode</t>
+          <t>Flexible/rate-table billing</t>
         </is>
       </c>
       <c r="D68" s="5" t="inlineStr">
@@ -2798,29 +2798,29 @@
       </c>
       <c r="E68" s="6" t="inlineStr">
         <is>
-          <t>Phase 9</t>
+          <t>Phase 8 follow-up</t>
         </is>
       </c>
       <c r="F68" s="6" t="inlineStr">
         <is>
-          <t>As a hub dispatcher during the pilot, I want to preview the optimizer's proposed plan and override it if needed, so that I can build trust in autonomous dispatch before relying on it fully.</t>
+          <t>As a client with orders of very different sizes, I want billing that can reflect piece count, weight, or mileage, not just a flat per-drop rate, so that pricing matches the actual cost of serving my orders.</t>
         </is>
       </c>
     </row>
     <row r="69">
       <c r="A69" s="7" t="inlineStr">
         <is>
-          <t>I1</t>
+          <t>F6</t>
         </is>
       </c>
       <c r="B69" s="8" t="inlineStr">
         <is>
-          <t>Intelligence layer</t>
+          <t>Competitive gaps</t>
         </is>
       </c>
       <c r="C69" s="8" t="inlineStr">
         <is>
-          <t>Ground-truth event capture</t>
+          <t>Real-time mid-route re-optimization</t>
         </is>
       </c>
       <c r="D69" s="7" t="inlineStr">
@@ -2830,29 +2830,29 @@
       </c>
       <c r="E69" s="8" t="inlineStr">
         <is>
-          <t>Phase 10 (pre-pilot)</t>
+          <t>Phase 4 (needs E1)</t>
         </is>
       </c>
       <c r="F69" s="8" t="inlineStr">
         <is>
-          <t>As the Learning Loop, I want real delivered/arrived timestamps and decline/hold-release data captured, so that there's actual ground truth to learn from instead of a proxy that was never meant for this.</t>
+          <t>As a hub dispatcher, I want the optimizer to re-sequence an in-progress route when conditions change, so that a driver isn't stuck following a plan that's gone stale since the last cycle.</t>
         </is>
       </c>
     </row>
     <row r="70">
       <c r="A70" s="5" t="inlineStr">
         <is>
-          <t>I2</t>
+          <t>F7</t>
         </is>
       </c>
       <c r="B70" s="6" t="inlineStr">
         <is>
-          <t>Intelligence layer</t>
+          <t>Competitive gaps</t>
         </is>
       </c>
       <c r="C70" s="6" t="inlineStr">
         <is>
-          <t>Rule review &amp; promotion flow</t>
+          <t>Client- and ops-facing analytics dashboards</t>
         </is>
       </c>
       <c r="D70" s="5" t="inlineStr">
@@ -2862,29 +2862,29 @@
       </c>
       <c r="E70" s="6" t="inlineStr">
         <is>
-          <t>Phase 10 (pre-pilot)</t>
+          <t>Phase 10 (folds into I4)</t>
         </is>
       </c>
       <c r="F70" s="6" t="inlineStr">
         <is>
-          <t>As a hub ops manager, I want to review and approve or dismiss a proposed rule change from the Learning Loop, so that per-shop overrides get vetted by a person before they take effect.</t>
+          <t>As a client company, I want to see my own on-time rate, volume, and cost trend in the portal, so that I have concrete proof of the value of switching to per-drop pricing with LMX.</t>
         </is>
       </c>
     </row>
     <row r="71">
       <c r="A71" s="7" t="inlineStr">
         <is>
-          <t>I3</t>
+          <t>F8</t>
         </is>
       </c>
       <c r="B71" s="8" t="inlineStr">
         <is>
-          <t>Intelligence layer</t>
+          <t>Competitive gaps</t>
         </is>
       </c>
       <c r="C71" s="8" t="inlineStr">
         <is>
-          <t>Broaden the annotation vocabulary</t>
+          <t>White-label / multi-brand portal theming</t>
         </is>
       </c>
       <c r="D71" s="7" t="inlineStr">
@@ -2894,209 +2894,529 @@
       </c>
       <c r="E71" s="8" t="inlineStr">
         <is>
-          <t>Phase 10 (pre-pilot)</t>
+          <t>Phase 8 follow-up</t>
         </is>
       </c>
       <c r="F71" s="8" t="inlineStr">
         <is>
-          <t>As a driver, I want to flag more than just hold-window issues (parking, gate codes, shop prep slowness), so that what I know about a shop becomes part of the system instead of staying in my head.</t>
+          <t>As a reselling partner, I want the client portal to carry my own brand, so that my customers experience it as part of my business, not a visibly third-party tool.</t>
         </is>
       </c>
     </row>
     <row r="72">
       <c r="A72" s="5" t="inlineStr">
         <is>
-          <t>I4</t>
+          <t>F9</t>
         </is>
       </c>
       <c r="B72" s="6" t="inlineStr">
         <is>
-          <t>Intelligence layer</t>
+          <t>Competitive gaps</t>
         </is>
       </c>
       <c r="C72" s="6" t="inlineStr">
         <is>
-          <t>Descriptive analytics on the captured truth</t>
-        </is>
-      </c>
-      <c r="D72" s="5" t="inlineStr">
-        <is>
-          <t>Open</t>
+          <t>Hybrid gig-fleet overflow dispatch</t>
+        </is>
+      </c>
+      <c r="D72" s="13" t="inlineStr">
+        <is>
+          <t>Superseded -&gt; reinstated as P7</t>
         </is>
       </c>
       <c r="E72" s="6" t="inlineStr">
         <is>
-          <t>Phase 10 (during/after pilot)</t>
+          <t>-</t>
         </is>
       </c>
       <c r="F72" s="6" t="inlineStr">
         <is>
-          <t>As a hub ops manager, I want DPH, SLA hit rate, and hold-window effectiveness reported per driver/hub/day, so that I can see how the operation is actually performing, not just whether the day went fine.</t>
+          <t>Superseded: see P7 for the current, generalized version of this story (LMX leadership routing to the cheapest eligible capacity, including gig couriers).</t>
         </is>
       </c>
     </row>
     <row r="73">
       <c r="A73" s="7" t="inlineStr">
         <is>
-          <t>I5</t>
+          <t>F10</t>
         </is>
       </c>
       <c r="B73" s="8" t="inlineStr">
         <is>
-          <t>Intelligence layer</t>
+          <t>Competitive gaps</t>
         </is>
       </c>
       <c r="C73" s="8" t="inlineStr">
         <is>
-          <t>Calibration from data</t>
+          <t>A real path to SOC 2 (or equivalent) certification</t>
         </is>
       </c>
       <c r="D73" s="7" t="inlineStr">
         <is>
-          <t>Open (=E2/E5/E9/E10)</t>
+          <t>Open</t>
         </is>
       </c>
       <c r="E73" s="8" t="inlineStr">
         <is>
-          <t>Phase 10 (during/after pilot)</t>
+          <t>Phase 5</t>
         </is>
       </c>
       <c r="F73" s="8" t="inlineStr">
         <is>
-          <t>As LMX leadership, I want skip penalties, hold windows, and the DPH figure retuned from real data, so that every placeholder number gets replaced with something proven.</t>
+          <t>As an enterprise client's security team, I want to see a SOC 2 report before signing, so that I have independent assurance LMX handles data and access responsibly.</t>
         </is>
       </c>
     </row>
     <row r="74">
       <c r="A74" s="5" t="inlineStr">
         <is>
-          <t>I6</t>
+          <t>F11</t>
         </is>
       </c>
       <c r="B74" s="6" t="inlineStr">
         <is>
-          <t>Intelligence layer</t>
+          <t>Competitive gaps</t>
         </is>
       </c>
       <c r="C74" s="6" t="inlineStr">
         <is>
-          <t>Predictive models</t>
+          <t>SSO/SAML for ops and client logins</t>
         </is>
       </c>
       <c r="D74" s="5" t="inlineStr">
         <is>
-          <t>Open (data-gated)</t>
+          <t>Open</t>
         </is>
       </c>
       <c r="E74" s="6" t="inlineStr">
         <is>
-          <t>Phase 10 (later)</t>
+          <t>Phase 5</t>
         </is>
       </c>
       <c r="F74" s="6" t="inlineStr">
         <is>
-          <t>As a hub dispatcher, I want the optimizer to use predicted ETAs and per-shop service times instead of static estimates, so that routes reflect what's actually likely to happen, not a fixed assumption.</t>
+          <t>As an enterprise client's IT admin, I want to enforce SSO for anyone accessing the portal, so that portal access follows the same identity policy as the rest of my company's tools.</t>
         </is>
       </c>
     </row>
     <row r="75">
       <c r="A75" s="7" t="inlineStr">
         <is>
-          <t>I7</t>
+          <t>F12</t>
         </is>
       </c>
       <c r="B75" s="8" t="inlineStr">
         <is>
-          <t>Intelligence layer</t>
+          <t>Competitive gaps</t>
         </is>
       </c>
       <c r="C75" s="8" t="inlineStr">
         <is>
-          <t>Ops copilot</t>
+          <t>Network/territory optimization tooling</t>
         </is>
       </c>
       <c r="D75" s="7" t="inlineStr">
         <is>
-          <t>Open (needs LLM API key)</t>
+          <t>Open</t>
         </is>
       </c>
       <c r="E75" s="8" t="inlineStr">
         <is>
-          <t>Phase 10 (later)</t>
+          <t>Later, multi-hub</t>
         </is>
       </c>
       <c r="F75" s="8" t="inlineStr">
         <is>
-          <t>As a hub ops manager, I want to ask a natural-language question like 'why was yesterday slow?' and get a real answer from the system's own data, so that I don't have to manually dig through dashboards to explain a bad day.</t>
+          <t>As LMX leadership planning a second or third hub, I want tooling to redesign depot/zone boundaries, so that expansion decisions are based on a real optimization model instead of intuition.</t>
         </is>
       </c>
     </row>
     <row r="76">
       <c r="A76" s="5" t="inlineStr">
         <is>
-          <t>T1</t>
+          <t>F13</t>
         </is>
       </c>
       <c r="B76" s="6" t="inlineStr">
         <is>
-          <t>Testing/process</t>
+          <t>Competitive gaps</t>
         </is>
       </c>
       <c r="C76" s="6" t="inlineStr">
         <is>
-          <t>Load/performance test against the design budget</t>
-        </is>
-      </c>
-      <c r="D76" s="10" t="inlineStr">
-        <is>
-          <t>Done</t>
+          <t>Ratings &amp; feedback capture</t>
+        </is>
+      </c>
+      <c r="D76" s="5" t="inlineStr">
+        <is>
+          <t>Open</t>
         </is>
       </c>
       <c r="E76" s="6" t="inlineStr">
         <is>
-          <t>Phase 9</t>
+          <t>Phase 8 follow-up</t>
         </is>
       </c>
       <c r="F76" s="6" t="inlineStr">
         <is>
-          <t>As the engineering team, I want the optimizer load-tested against the design budget (20 drivers/100 orders/&lt;5s), so that we know the dispatch cycle holds up before it's carrying real orders.</t>
+          <t>As a shop after a delivery, I want to leave a quick rating and comment, so that LMX knows how the delivery actually went, not just whether the status says completed.</t>
         </is>
       </c>
     </row>
     <row r="77">
       <c r="A77" s="7" t="inlineStr">
         <is>
+          <t>F14</t>
+        </is>
+      </c>
+      <c r="B77" s="8" t="inlineStr">
+        <is>
+          <t>Competitive gaps</t>
+        </is>
+      </c>
+      <c r="C77" s="8" t="inlineStr">
+        <is>
+          <t>Orchestrator route-preview / shadow mode</t>
+        </is>
+      </c>
+      <c r="D77" s="7" t="inlineStr">
+        <is>
+          <t>Open</t>
+        </is>
+      </c>
+      <c r="E77" s="8" t="inlineStr">
+        <is>
+          <t>Phase 9</t>
+        </is>
+      </c>
+      <c r="F77" s="8" t="inlineStr">
+        <is>
+          <t>As a hub dispatcher during the pilot, I want to preview the optimizer's proposed plan and override it if needed, so that I can build trust in autonomous dispatch before relying on it fully.</t>
+        </is>
+      </c>
+    </row>
+    <row r="78">
+      <c r="A78" s="5" t="inlineStr">
+        <is>
+          <t>I1</t>
+        </is>
+      </c>
+      <c r="B78" s="6" t="inlineStr">
+        <is>
+          <t>Intelligence layer</t>
+        </is>
+      </c>
+      <c r="C78" s="6" t="inlineStr">
+        <is>
+          <t>Ground-truth event capture</t>
+        </is>
+      </c>
+      <c r="D78" s="5" t="inlineStr">
+        <is>
+          <t>Open</t>
+        </is>
+      </c>
+      <c r="E78" s="6" t="inlineStr">
+        <is>
+          <t>Phase 10 (pre-pilot)</t>
+        </is>
+      </c>
+      <c r="F78" s="6" t="inlineStr">
+        <is>
+          <t>As the Learning Loop, I want real delivered/arrived timestamps and decline/hold-release data captured, so that there's actual ground truth to learn from instead of a proxy that was never meant for this.</t>
+        </is>
+      </c>
+    </row>
+    <row r="79">
+      <c r="A79" s="7" t="inlineStr">
+        <is>
+          <t>I8</t>
+        </is>
+      </c>
+      <c r="B79" s="8" t="inlineStr">
+        <is>
+          <t>Intelligence layer</t>
+        </is>
+      </c>
+      <c r="C79" s="8" t="inlineStr">
+        <is>
+          <t>Manual capture of non-default training situations</t>
+        </is>
+      </c>
+      <c r="D79" s="7" t="inlineStr">
+        <is>
+          <t>Open</t>
+        </is>
+      </c>
+      <c r="E79" s="8" t="inlineStr">
+        <is>
+          <t>Phase 3.5 / Phase 9</t>
+        </is>
+      </c>
+      <c r="F79" s="8" t="inlineStr">
+        <is>
+          <t>As whoever runs Hub 1 operations, I want a checklist of the training situations that aren't captured automatically - the paired access-note comparison, the dispatcher gut-call log, the scaffold-era call tally, the shadow divergence pairs - so that the third of the training matrix that needs a human to write it down actually gets written down, including two things only capturable before cutover.</t>
+        </is>
+      </c>
+    </row>
+    <row r="80">
+      <c r="A80" s="5" t="inlineStr">
+        <is>
+          <t>I2</t>
+        </is>
+      </c>
+      <c r="B80" s="6" t="inlineStr">
+        <is>
+          <t>Intelligence layer</t>
+        </is>
+      </c>
+      <c r="C80" s="6" t="inlineStr">
+        <is>
+          <t>Rule review &amp; promotion flow</t>
+        </is>
+      </c>
+      <c r="D80" s="5" t="inlineStr">
+        <is>
+          <t>Open</t>
+        </is>
+      </c>
+      <c r="E80" s="6" t="inlineStr">
+        <is>
+          <t>Phase 10 (pre-pilot)</t>
+        </is>
+      </c>
+      <c r="F80" s="6" t="inlineStr">
+        <is>
+          <t>As a hub ops manager, I want to review and approve or dismiss a proposed rule change from the Learning Loop, so that per-shop overrides get vetted by a person before they take effect.</t>
+        </is>
+      </c>
+    </row>
+    <row r="81">
+      <c r="A81" s="7" t="inlineStr">
+        <is>
+          <t>I3</t>
+        </is>
+      </c>
+      <c r="B81" s="8" t="inlineStr">
+        <is>
+          <t>Intelligence layer</t>
+        </is>
+      </c>
+      <c r="C81" s="8" t="inlineStr">
+        <is>
+          <t>Broaden the annotation vocabulary</t>
+        </is>
+      </c>
+      <c r="D81" s="7" t="inlineStr">
+        <is>
+          <t>Open</t>
+        </is>
+      </c>
+      <c r="E81" s="8" t="inlineStr">
+        <is>
+          <t>Phase 10 (pre-pilot)</t>
+        </is>
+      </c>
+      <c r="F81" s="8" t="inlineStr">
+        <is>
+          <t>As a driver, I want to flag more than just hold-window issues (parking, gate codes, shop prep slowness), so that what I know about a shop becomes part of the system instead of staying in my head.</t>
+        </is>
+      </c>
+    </row>
+    <row r="82">
+      <c r="A82" s="5" t="inlineStr">
+        <is>
+          <t>I4</t>
+        </is>
+      </c>
+      <c r="B82" s="6" t="inlineStr">
+        <is>
+          <t>Intelligence layer</t>
+        </is>
+      </c>
+      <c r="C82" s="6" t="inlineStr">
+        <is>
+          <t>Descriptive analytics on the captured truth</t>
+        </is>
+      </c>
+      <c r="D82" s="5" t="inlineStr">
+        <is>
+          <t>Open</t>
+        </is>
+      </c>
+      <c r="E82" s="6" t="inlineStr">
+        <is>
+          <t>Phase 10 (during/after pilot)</t>
+        </is>
+      </c>
+      <c r="F82" s="6" t="inlineStr">
+        <is>
+          <t>As a hub ops manager, I want DPH, SLA hit rate, and hold-window effectiveness reported per driver/hub/day, so that I can see how the operation is actually performing, not just whether the day went fine.</t>
+        </is>
+      </c>
+    </row>
+    <row r="83">
+      <c r="A83" s="7" t="inlineStr">
+        <is>
+          <t>I5</t>
+        </is>
+      </c>
+      <c r="B83" s="8" t="inlineStr">
+        <is>
+          <t>Intelligence layer</t>
+        </is>
+      </c>
+      <c r="C83" s="8" t="inlineStr">
+        <is>
+          <t>Calibration from data</t>
+        </is>
+      </c>
+      <c r="D83" s="7" t="inlineStr">
+        <is>
+          <t>Open (=E2/E5/E9/E10)</t>
+        </is>
+      </c>
+      <c r="E83" s="8" t="inlineStr">
+        <is>
+          <t>Phase 10 (during/after pilot)</t>
+        </is>
+      </c>
+      <c r="F83" s="8" t="inlineStr">
+        <is>
+          <t>As LMX leadership, I want skip penalties, hold windows, and the DPH figure retuned from real data, so that every placeholder number gets replaced with something proven.</t>
+        </is>
+      </c>
+    </row>
+    <row r="84">
+      <c r="A84" s="5" t="inlineStr">
+        <is>
+          <t>I6</t>
+        </is>
+      </c>
+      <c r="B84" s="6" t="inlineStr">
+        <is>
+          <t>Intelligence layer</t>
+        </is>
+      </c>
+      <c r="C84" s="6" t="inlineStr">
+        <is>
+          <t>Predictive models</t>
+        </is>
+      </c>
+      <c r="D84" s="5" t="inlineStr">
+        <is>
+          <t>Open (data-gated)</t>
+        </is>
+      </c>
+      <c r="E84" s="6" t="inlineStr">
+        <is>
+          <t>Phase 10 (later)</t>
+        </is>
+      </c>
+      <c r="F84" s="6" t="inlineStr">
+        <is>
+          <t>As a hub dispatcher, I want the optimizer to use predicted ETAs and per-shop service times instead of static estimates, so that routes reflect what's actually likely to happen, not a fixed assumption.</t>
+        </is>
+      </c>
+    </row>
+    <row r="85">
+      <c r="A85" s="7" t="inlineStr">
+        <is>
+          <t>I7</t>
+        </is>
+      </c>
+      <c r="B85" s="8" t="inlineStr">
+        <is>
+          <t>Intelligence layer</t>
+        </is>
+      </c>
+      <c r="C85" s="8" t="inlineStr">
+        <is>
+          <t>Ops copilot</t>
+        </is>
+      </c>
+      <c r="D85" s="7" t="inlineStr">
+        <is>
+          <t>Open (needs LLM API key)</t>
+        </is>
+      </c>
+      <c r="E85" s="8" t="inlineStr">
+        <is>
+          <t>Phase 10 (later)</t>
+        </is>
+      </c>
+      <c r="F85" s="8" t="inlineStr">
+        <is>
+          <t>As a hub ops manager, I want to ask a natural-language question like 'why was yesterday slow?' and get a real answer from the system's own data, so that I don't have to manually dig through dashboards to explain a bad day.</t>
+        </is>
+      </c>
+    </row>
+    <row r="86">
+      <c r="A86" s="5" t="inlineStr">
+        <is>
+          <t>T1</t>
+        </is>
+      </c>
+      <c r="B86" s="6" t="inlineStr">
+        <is>
+          <t>Testing/process</t>
+        </is>
+      </c>
+      <c r="C86" s="6" t="inlineStr">
+        <is>
+          <t>Load/performance test against the design budget</t>
+        </is>
+      </c>
+      <c r="D86" s="10" t="inlineStr">
+        <is>
+          <t>Done</t>
+        </is>
+      </c>
+      <c r="E86" s="6" t="inlineStr">
+        <is>
+          <t>Phase 9</t>
+        </is>
+      </c>
+      <c r="F86" s="6" t="inlineStr">
+        <is>
+          <t>As the engineering team, I want the optimizer load-tested against the design budget (20 drivers/100 orders/&lt;5s), so that we know the dispatch cycle holds up before it's carrying real orders.</t>
+        </is>
+      </c>
+    </row>
+    <row r="87">
+      <c r="A87" s="7" t="inlineStr">
+        <is>
           <t>T2</t>
         </is>
       </c>
-      <c r="B77" s="8" t="inlineStr">
+      <c r="B87" s="8" t="inlineStr">
         <is>
           <t>Testing/process</t>
         </is>
       </c>
-      <c r="C77" s="8" t="inlineStr">
+      <c r="C87" s="8" t="inlineStr">
         <is>
           <t>Local sandbox can't fully exercise Redis rate limiting</t>
         </is>
       </c>
-      <c r="D77" s="7" t="inlineStr">
+      <c r="D87" s="7" t="inlineStr">
         <is>
           <t>Documented, not a bug</t>
         </is>
       </c>
-      <c r="E77" s="8" t="inlineStr">
+      <c r="E87" s="8" t="inlineStr">
         <is>
           <t>-</t>
         </is>
       </c>
-      <c r="F77" s="8" t="inlineStr">
+      <c r="F87" s="8" t="inlineStr">
         <is>
           <t>As the engineering team, I want it documented that the sandbox's test Redis can't exercise EXPIRE...NX the way production Redis does, so that this known limitation doesn't get 'rediscovered' and mistaken for a real bug.</t>
         </is>
       </c>
     </row>
   </sheetData>
-  <autoFilter ref="A1:F77"/>
+  <autoFilter ref="A1:F87"/>
   <pageMargins left="0.75" right="0.75" top="1" bottom="1" header="0.5" footer="0.5"/>
 </worksheet>
 </file>
</xml_diff>